<commit_message>
Fix: Data Validation per Named Ranges statt inline (Excel 255-Char-Limit)
- REKO-Dropdown war 420 Zeichen lang -> Excel verwarf Datenüberprüfung
- Dropdown-Listen (Namen, REKO, Kategorien) jetzt im Hilfslisten-Sheet
- Named Ranges (NamenListe, REKOListe, KatListe) als Referenz
- Datums-Validierung entfernt (verursachte zusätzliche Kompatibilitätsprobleme)
- Keine "defekte Datei"-Warnung mehr beim Öffnen

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/LARIS_2026.xlsx
+++ b/LARIS_2026.xlsx
@@ -23,6 +23,9 @@
     <sheet name="Hilfslisten" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
+    <definedName name="NamenListe">Hilfslisten!$F$23:$F$39</definedName>
+    <definedName name="REKOListe">Hilfslisten!$H$23:$H$40</definedName>
+    <definedName name="KatListe">Hilfslisten!$J$23:$J$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sekretariat'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Sekretariat'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EDV'!$A$4:$L$57</definedName>
@@ -2714,18 +2717,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -3774,18 +3774,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -4864,18 +4861,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -5032,13 +5026,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
     <col width="40" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -5361,6 +5358,254 @@
         </is>
       </c>
       <c r="D18" s="69" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="F22" s="38" t="inlineStr">
+        <is>
+          <t>Dropdown: Namen</t>
+        </is>
+      </c>
+      <c r="H22" s="38" t="inlineStr">
+        <is>
+          <t>Dropdown: REKO</t>
+        </is>
+      </c>
+      <c r="J22" s="38" t="inlineStr">
+        <is>
+          <t>Dropdown: Kategorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="F23" s="37" t="inlineStr">
+        <is>
+          <t>Breig</t>
+        </is>
+      </c>
+      <c r="H23" s="37" t="inlineStr">
+        <is>
+          <t>REKO</t>
+        </is>
+      </c>
+      <c r="J23" s="37" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="F24" s="37" t="inlineStr">
+        <is>
+          <t>Dr. Vitez</t>
+        </is>
+      </c>
+      <c r="H24" s="37" t="inlineStr">
+        <is>
+          <t>Nicht erforderlich</t>
+        </is>
+      </c>
+      <c r="J24" s="37" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="F25" s="37" t="inlineStr">
+        <is>
+          <t>Dr.Frei</t>
+        </is>
+      </c>
+      <c r="H25" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Dr.Frei</t>
+        </is>
+      </c>
+      <c r="J25" s="37" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="F26" s="37" t="inlineStr">
+        <is>
+          <t>Dr.Schmidt</t>
+        </is>
+      </c>
+      <c r="H26" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Dr.Schmidt</t>
+        </is>
+      </c>
+      <c r="J26" s="37" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="F27" s="37" t="inlineStr">
+        <is>
+          <t>Goepfrich</t>
+        </is>
+      </c>
+      <c r="H27" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Dr. Vitez</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="F28" s="37" t="inlineStr">
+        <is>
+          <t>Göpfrich</t>
+        </is>
+      </c>
+      <c r="H28" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Breig</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="F29" s="37" t="inlineStr">
+        <is>
+          <t>Jochim</t>
+        </is>
+      </c>
+      <c r="H29" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Krempl</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="F30" s="37" t="inlineStr">
+        <is>
+          <t>Krempl</t>
+        </is>
+      </c>
+      <c r="H30" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Siebert</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="F31" s="37" t="inlineStr">
+        <is>
+          <t>Müller-Horn</t>
+        </is>
+      </c>
+      <c r="H31" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Putschler</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="F32" s="37" t="inlineStr">
+        <is>
+          <t>Putschler</t>
+        </is>
+      </c>
+      <c r="H32" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Jochim</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="F33" s="37" t="inlineStr">
+        <is>
+          <t>Radimersky</t>
+        </is>
+      </c>
+      <c r="H33" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Zuber</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="F34" s="37" t="inlineStr">
+        <is>
+          <t>Schmidt</t>
+        </is>
+      </c>
+      <c r="H34" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Göpfrich</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="F35" s="37" t="inlineStr">
+        <is>
+          <t>Siebert</t>
+        </is>
+      </c>
+      <c r="H35" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Zeller</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="F36" s="37" t="inlineStr">
+        <is>
+          <t>Wunsch</t>
+        </is>
+      </c>
+      <c r="H36" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Schmidt</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="F37" s="37" t="inlineStr">
+        <is>
+          <t>Zeller</t>
+        </is>
+      </c>
+      <c r="H37" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Zieger-Buchta</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="F38" s="37" t="inlineStr">
+        <is>
+          <t>Zieger-Buchta</t>
+        </is>
+      </c>
+      <c r="H38" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Müller-Horn</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="F39" s="37" t="inlineStr">
+        <is>
+          <t>Zuber</t>
+        </is>
+      </c>
+      <c r="H39" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Radimersky</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="H40" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Wunsch</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -6998,18 +7243,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -8194,18 +8436,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -9354,18 +9593,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -10470,18 +10706,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -11762,18 +11995,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -12868,18 +13098,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
@@ -14176,18 +14403,15 @@
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="4">
+  <dataValidations count="3">
     <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>"Breig,Dr. Vitez,Dr.Frei,Dr.Schmidt,Goepfrich,Göpfrich,Jochim,Krempl,Müller-Horn,Putschler,Radimersky,Schmidt,Siebert,Wunsch,Zeller,Zieger-Buchta,Zuber"</formula1>
+      <formula1>=NamenListe</formula1>
     </dataValidation>
     <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>"A,B,C,D"</formula1>
+      <formula1>=KatListe</formula1>
     </dataValidation>
     <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>"REKO,Nicht erforderlich,Besprochen mit  Dr.Frei,Besprochen mit  Dr.Schmidt,Besprochen mit  Dr. Vitez,Besprochen mit  Breig,Besprochen mit  Krempl,Besprochen mit  Siebert,Besprochen mit  Putschler,Besprochen mit  Jochim,Besprochen mit  Zuber,Besprochen mit  Göpfrich,Besprochen mit  Zeller,Besprochen mit  Schmidt,Besprochen mit  Zieger-Buchta,Besprochen mit  Müller-Horn,Besprochen mit  Radimersky,Besprochen mit  Wunsch"</formula1>
-    </dataValidation>
-    <dataValidation sqref="B5:B504 E5:E504 H5:H504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiges Datum" error="Bitte ein gültiges Datum eingeben (TT.MM.JJJJ oder TT.MM.JJJJ HH:MM)" promptTitle="Datum" prompt="Datum eingeben: TT.MM.JJJJ" type="date" operator="greaterThan">
-      <formula1>2024-01-01</formula1>
+      <formula1>=REKOListe</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>

<commit_message>
Sauberer Neustart: 2025-Daten entfernt, Getriebewerk weg, Namen bereinigt
- Alle Meldungsdaten aus 2025 entfernt (wird jährlich archiviert)
- Getriebewerk-Bereich komplett entfernt (9 statt 10 Bereiche)
- "Goepfrich" Duplikat entfernt -> nur noch "Göpfrich" im Dropdown
- RTW & MPG Leiter korrigiert auf "Göpfrich"
- Fehlende REKO-Einträge ergänzt (Jochim, Wunsch)
- Dr.Frei Funktion von "Leiter Getriebewerk" auf "Arzt" geändert

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/LARIS_2026.xlsx
+++ b/LARIS_2026.xlsx
@@ -17,35 +17,32 @@
     <sheet name="Organisation Ambulanz" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Ablauf&amp;Prozessprobleme" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="BGF" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Getriebewerk" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Hygiene" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Fehlerkategorien" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Hilfslisten" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Hygiene" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Fehlerkategorien" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Hilfslisten" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
-    <definedName name="NamenListe">Hilfslisten!$F$23:$F$39</definedName>
-    <definedName name="REKOListe">Hilfslisten!$H$23:$H$40</definedName>
+    <definedName name="NamenListe">Hilfslisten!$F$23:$F$38</definedName>
+    <definedName name="REKOListe">Hilfslisten!$H$23:$H$42</definedName>
     <definedName name="KatListe">Hilfslisten!$J$23:$J$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sekretariat'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Sekretariat'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EDV'!$A$4:$L$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EDV'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'EDV'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Med.&amp;Verbr.-stoff'!$A$4:$L$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Med.&amp;Verbr.-stoff'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Med.&amp;Verbr.-stoff'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'WD-Fzg &amp; Schutzkleidg'!$A$4:$L$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'WD-Fzg &amp; Schutzkleidg'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'WD-Fzg &amp; Schutzkleidg'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'RTW &amp; MPG'!$A$4:$L$59</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'RTW &amp; MPG'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'RTW &amp; MPG'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Organisation Ambulanz'!$A$4:$L$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Organisation Ambulanz'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Organisation Ambulanz'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Ablauf&amp;Prozessprobleme'!$A$4:$L$60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Ablauf&amp;Prozessprobleme'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Ablauf&amp;Prozessprobleme'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'BGF'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'BGF'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Getriebewerk'!$A$4:$L$54</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Getriebewerk'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Hygiene'!$A$4:$L$55</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="11">'Hygiene'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Hygiene'!$A$4:$L$54</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="10">'Hygiene'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -53,9 +50,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD.MM.YYYY HH:MM"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="23">
     <font>
@@ -342,7 +338,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="70">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -454,9 +450,6 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -965,7 +958,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:L27"/>
+  <dimension ref="B1:L26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -998,7 +991,7 @@
         </is>
       </c>
       <c r="D4" s="3">
-        <f>C17</f>
+        <f>C16</f>
         <v/>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1007,7 +1000,7 @@
         </is>
       </c>
       <c r="G4" s="4">
-        <f>D17</f>
+        <f>D16</f>
         <v/>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -1016,7 +1009,7 @@
         </is>
       </c>
       <c r="J4" s="5">
-        <f>E17</f>
+        <f>E16</f>
         <v/>
       </c>
     </row>
@@ -1275,7 +1268,7 @@
       <c r="K11" s="11" t="n"/>
       <c r="L11" s="12" t="inlineStr">
         <is>
-          <t>Goepfrich</t>
+          <t>Göpfrich</t>
         </is>
       </c>
     </row>
@@ -1408,15 +1401,15 @@
     <row r="15">
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Getriebewerk</t>
+          <t>Hygiene</t>
         </is>
       </c>
       <c r="C15" s="8">
-        <f>COUNTA('Getriebewerk'!B5:B504)</f>
+        <f>COUNTA('Hygiene'!B5:B504)</f>
         <v/>
       </c>
       <c r="D15" s="9">
-        <f>COUNTA('Getriebewerk'!H5:H504)</f>
+        <f>COUNTA('Hygiene'!H5:H504)</f>
         <v/>
       </c>
       <c r="E15" s="10">
@@ -1425,214 +1418,172 @@
       </c>
       <c r="F15" s="11" t="n"/>
       <c r="G15" s="12">
-        <f>COUNTIF('Getriebewerk'!J5:J504,"A")</f>
+        <f>COUNTIF('Hygiene'!J5:J504,"A")</f>
         <v/>
       </c>
       <c r="H15" s="12">
-        <f>COUNTIF('Getriebewerk'!J5:J504,"B")</f>
+        <f>COUNTIF('Hygiene'!J5:J504,"B")</f>
         <v/>
       </c>
       <c r="I15" s="12">
-        <f>COUNTIF('Getriebewerk'!J5:J504,"C")</f>
+        <f>COUNTIF('Hygiene'!J5:J504,"C")</f>
         <v/>
       </c>
       <c r="J15" s="12">
-        <f>COUNTIF('Getriebewerk'!J5:J504,"D")</f>
+        <f>COUNTIF('Hygiene'!J5:J504,"D")</f>
         <v/>
       </c>
       <c r="K15" s="11" t="n"/>
       <c r="L15" s="12" t="inlineStr">
         <is>
-          <t>Dr.Frei</t>
+          <t>Wunsch</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Hygiene</t>
-        </is>
-      </c>
-      <c r="C16" s="14">
-        <f>COUNTA('Hygiene'!B5:B504)</f>
-        <v/>
-      </c>
-      <c r="D16" s="15">
-        <f>COUNTA('Hygiene'!H5:H504)</f>
-        <v/>
-      </c>
-      <c r="E16" s="16">
-        <f>C16-D16</f>
-        <v/>
-      </c>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="18">
-        <f>COUNTIF('Hygiene'!J5:J504,"A")</f>
-        <v/>
-      </c>
-      <c r="H16" s="18">
-        <f>COUNTIF('Hygiene'!J5:J504,"B")</f>
-        <v/>
-      </c>
-      <c r="I16" s="18">
-        <f>COUNTIF('Hygiene'!J5:J504,"C")</f>
-        <v/>
-      </c>
-      <c r="J16" s="18">
-        <f>COUNTIF('Hygiene'!J5:J504,"D")</f>
-        <v/>
-      </c>
-      <c r="K16" s="17" t="n"/>
-      <c r="L16" s="18" t="inlineStr">
-        <is>
-          <t>Wunsch</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="19" t="inlineStr">
+      <c r="B16" s="19" t="inlineStr">
         <is>
           <t>GESAMT</t>
         </is>
       </c>
-      <c r="C17" s="19">
-        <f>SUM(C7:C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="19">
-        <f>SUM(D7:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="19">
-        <f>SUM(E7:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="20" t="n"/>
-      <c r="G17" s="19">
-        <f>SUM(G7:G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="19">
-        <f>SUM(H7:H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="19">
-        <f>SUM(I7:I16)</f>
-        <v/>
-      </c>
-      <c r="J17" s="19">
-        <f>SUM(J7:J16)</f>
-        <v/>
-      </c>
-      <c r="K17" s="20" t="n"/>
-      <c r="L17" s="21" t="n"/>
+      <c r="C16" s="19">
+        <f>SUM(C7:C15)</f>
+        <v/>
+      </c>
+      <c r="D16" s="19">
+        <f>SUM(D7:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="19">
+        <f>SUM(E7:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="20" t="n"/>
+      <c r="G16" s="19">
+        <f>SUM(G7:G15)</f>
+        <v/>
+      </c>
+      <c r="H16" s="19">
+        <f>SUM(H7:H15)</f>
+        <v/>
+      </c>
+      <c r="I16" s="19">
+        <f>SUM(I7:I15)</f>
+        <v/>
+      </c>
+      <c r="J16" s="19">
+        <f>SUM(J7:J15)</f>
+        <v/>
+      </c>
+      <c r="K16" s="20" t="n"/>
+      <c r="L16" s="21" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Legende Farbmarkierungen in den Bereichs-Sheets:</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="B19" s="22" t="inlineStr">
-        <is>
-          <t>Legende Farbmarkierungen in den Bereichs-Sheets:</t>
+      <c r="B19" s="23" t="n"/>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>Nr.-Spalte blau</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr">
+        <is>
+          <t>Neue Meldung (letzte 7 Tage)</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="23" t="n"/>
+      <c r="B20" s="26" t="n"/>
       <c r="C20" s="24" t="inlineStr">
         <is>
-          <t>Nr.-Spalte blau</t>
+          <t>Zeile gelb</t>
         </is>
       </c>
       <c r="D20" s="25" t="inlineStr">
         <is>
-          <t>Neue Meldung (letzte 7 Tage)</t>
+          <t>Meldung offen (noch nicht erledigt)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="26" t="n"/>
+      <c r="B21" s="27" t="n"/>
       <c r="C21" s="24" t="inlineStr">
         <is>
-          <t>Zeile gelb</t>
+          <t>Zeile grün</t>
         </is>
       </c>
       <c r="D21" s="25" t="inlineStr">
         <is>
-          <t>Meldung offen (noch nicht erledigt)</t>
+          <t>Meldung erledigt</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="27" t="n"/>
+      <c r="B22" s="28" t="n"/>
       <c r="C22" s="24" t="inlineStr">
         <is>
-          <t>Zeile grün</t>
+          <t>Zeile rot</t>
         </is>
       </c>
       <c r="D22" s="25" t="inlineStr">
         <is>
-          <t>Meldung erledigt</t>
+          <t>Überfällig (&gt;14 Tage ohne Kenntnisnahme)</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="28" t="n"/>
+      <c r="B23" s="29" t="n"/>
       <c r="C23" s="24" t="inlineStr">
         <is>
-          <t>Zeile rot</t>
+          <t>Kategorie A</t>
         </is>
       </c>
       <c r="D23" s="25" t="inlineStr">
         <is>
-          <t>Überfällig (&gt;14 Tage ohne Kenntnisnahme)</t>
+          <t>Unsichere Handlung</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="29" t="n"/>
+      <c r="B24" s="30" t="n"/>
       <c r="C24" s="24" t="inlineStr">
         <is>
-          <t>Kategorie A</t>
+          <t>Kategorie B</t>
         </is>
       </c>
       <c r="D24" s="25" t="inlineStr">
         <is>
-          <t>Unsichere Handlung</t>
+          <t>Beinahefehler ohne Folgen</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="30" t="n"/>
+      <c r="B25" s="31" t="n"/>
       <c r="C25" s="24" t="inlineStr">
         <is>
-          <t>Kategorie B</t>
+          <t>Kategorie C</t>
         </is>
       </c>
       <c r="D25" s="25" t="inlineStr">
         <is>
-          <t>Beinahefehler ohne Folgen</t>
+          <t>Fehler mit leichten bis mittelschweren Folgen</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="31" t="n"/>
+      <c r="B26" s="32" t="n"/>
       <c r="C26" s="24" t="inlineStr">
         <is>
-          <t>Kategorie C</t>
+          <t>Kategorie D</t>
         </is>
       </c>
       <c r="D26" s="25" t="inlineStr">
-        <is>
-          <t>Fehler mit leichten bis mittelschweren Folgen</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="32" t="n"/>
-      <c r="C27" s="24" t="inlineStr">
-        <is>
-          <t>Kategorie D</t>
-        </is>
-      </c>
-      <c r="D27" s="25" t="inlineStr">
         <is>
           <t>Fehler mit gravierenden Folgen</t>
         </is>
@@ -1641,12 +1592,12 @@
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="E4:F4"/>
-    <mergeCell ref="D27:F27"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="D19:F19"/>
     <mergeCell ref="B1:J2"/>
     <mergeCell ref="D23:F23"/>
     <mergeCell ref="D22:F22"/>
     <mergeCell ref="D26:F26"/>
-    <mergeCell ref="B19:E19"/>
     <mergeCell ref="H4:I4"/>
     <mergeCell ref="D21:F21"/>
     <mergeCell ref="D25:F25"/>
@@ -1654,12 +1605,12 @@
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="D24:F24"/>
   </mergeCells>
-  <conditionalFormatting sqref="E7:E16">
+  <conditionalFormatting sqref="E7:E15">
     <cfRule type="cellIs" priority="1" operator="greaterThan" dxfId="0" stopIfTrue="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J7:J16">
+  <conditionalFormatting sqref="J7:J15">
     <cfRule type="cellIs" priority="2" operator="greaterThan" dxfId="1" stopIfTrue="0">
       <formula>0</formula>
     </cfRule>
@@ -1667,17 +1618,17 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G7:G16">
+  <conditionalFormatting sqref="G7:G15">
     <cfRule type="cellIs" priority="3" operator="greaterThan" dxfId="3" stopIfTrue="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H7:H16">
+  <conditionalFormatting sqref="H7:H15">
     <cfRule type="cellIs" priority="4" operator="greaterThan" dxfId="4" stopIfTrue="0">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7:I16">
+  <conditionalFormatting sqref="I7:I15">
     <cfRule type="cellIs" priority="5" operator="greaterThan" dxfId="5" stopIfTrue="0">
       <formula>0</formula>
     </cfRule>
@@ -2771,7 +2722,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="43" t="inlineStr">
         <is>
-          <t>Getriebewerk</t>
+          <t>Hygiene</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2766,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="49" t="inlineStr">
         <is>
-          <t>✉ Mail an Bereichsleiter: Dr.Frei (markus.frei@mercedes-benz.com)</t>
+          <t>✉ Mail an Bereichsleiter: Wunsch (Fabian.Wunsch@mercedes-benz.com)</t>
         </is>
       </c>
       <c r="H3" s="50" t="inlineStr">
@@ -3738,1093 +3689,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:L54"/>
-  <mergeCells count="4">
-    <mergeCell ref="H2:L2"/>
-    <mergeCell ref="H3:L3"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A3:G3"/>
-  </mergeCells>
-  <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
-      <formula>"A"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
-      <formula>"B"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
-      <formula>"C"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
-      <formula>"D"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
-      <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
-    </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
-      <formula>AND($B5&lt;&gt;"",$H5="")</formula>
-    </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
-      <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
-      <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="3">
-    <dataValidation sqref="C5:C504 F5:F504 I5:I504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültiger Name" error="Bitte einen Namen aus der Liste wählen" promptTitle="Mitarbeiter" prompt="Name auswählen" type="list">
-      <formula1>=NamenListe</formula1>
-    </dataValidation>
-    <dataValidation sqref="J5:J504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Kategorie" error="Bitte A, B, C oder D wählen" promptTitle="Fehlerkategorie" prompt="Kategorie wählen (A-D)" type="list">
-      <formula1>=KatListe</formula1>
-    </dataValidation>
-    <dataValidation sqref="L5:L504" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Ungültige Auswahl" error="Bitte aus der Liste wählen" promptTitle="REKO / Besprochen" prompt="Besprechungsart wählen" type="list">
-      <formula1>=REKOListe</formula1>
-    </dataValidation>
-  </dataValidations>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
-  </hyperlinks>
-  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;C&amp;10 LARIS - Getriebewerk</oddHeader>
-    <oddFooter>&amp;LWerksärztlicher Dienst Mercedes-Benz&amp;RSeite &amp;P von &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <tabColor rgb="000F3460"/>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:L55"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="10" max="10"/>
-    <col width="40" customWidth="1" min="11" max="11"/>
-    <col width="28" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="35" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
-        <is>
-          <t>Hygiene</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="55" customHeight="1">
-      <c r="A2" s="44" t="inlineStr">
-        <is>
-          <t>Meldungen:</t>
-        </is>
-      </c>
-      <c r="B2" s="45">
-        <f>COUNTA(B5:B504)</f>
-        <v/>
-      </c>
-      <c r="C2" s="44" t="inlineStr">
-        <is>
-          <t>Erledigt:</t>
-        </is>
-      </c>
-      <c r="D2" s="46">
-        <f>COUNTA(H5:H504)</f>
-        <v/>
-      </c>
-      <c r="E2" s="44" t="inlineStr">
-        <is>
-          <t>Offen:</t>
-        </is>
-      </c>
-      <c r="F2" s="47">
-        <f>B2-D2</f>
-        <v/>
-      </c>
-      <c r="H2" s="48" t="inlineStr">
-        <is>
-          <t>A = unsichere Handlung
-B = Beinahefehler ohne Folgen
-C = Fehler mit leichten bis mittelschweren Folgen
-D = Fehler mit gravierenden Folgen</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="49" t="inlineStr">
-        <is>
-          <t>✉ Mail an Bereichsleiter: Wunsch (Fabian.Wunsch@mercedes-benz.com)</t>
-        </is>
-      </c>
-      <c r="H3" s="50" t="inlineStr">
-        <is>
-          <t>BCC an: Putschler (walter.putschler@mercedes-benz.com)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="32" customHeight="1">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>Nr.</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>Meldung am</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Meldung durch</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Thema</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>Kenntnisnahme am</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>Kenntnisnahme durch</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>Massnahme</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>Erledigt am</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Erledigt durch</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>Kategorie</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>Info</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>In REKO oder Persönlich besprochen?</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="52" t="n">
-        <v>46055</v>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
-        <is>
-          <t>Wunsch</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>Hygiene Physikalische + Ruheraum, in letzter Zeit öfters schmutzige Liegen &amp; Schwämme noch am Gerät</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="n"/>
-      <c r="F5" s="51" t="inlineStr"/>
-      <c r="G5" s="53" t="inlineStr"/>
-      <c r="H5" s="52" t="n"/>
-      <c r="I5" s="51" t="inlineStr"/>
-      <c r="J5" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K5" s="53" t="inlineStr"/>
-      <c r="L5" s="53" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="51">
-        <f>IF(B6&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B6" s="52" t="n"/>
-      <c r="C6" s="51" t="n"/>
-      <c r="D6" s="53" t="n"/>
-      <c r="E6" s="52" t="n"/>
-      <c r="F6" s="51" t="n"/>
-      <c r="G6" s="53" t="n"/>
-      <c r="H6" s="52" t="n"/>
-      <c r="I6" s="51" t="n"/>
-      <c r="J6" s="51" t="n"/>
-      <c r="K6" s="53" t="n"/>
-      <c r="L6" s="53" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="51">
-        <f>IF(B7&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B7" s="52" t="n"/>
-      <c r="C7" s="51" t="n"/>
-      <c r="D7" s="53" t="n"/>
-      <c r="E7" s="52" t="n"/>
-      <c r="F7" s="51" t="n"/>
-      <c r="G7" s="53" t="n"/>
-      <c r="H7" s="52" t="n"/>
-      <c r="I7" s="51" t="n"/>
-      <c r="J7" s="51" t="n"/>
-      <c r="K7" s="53" t="n"/>
-      <c r="L7" s="53" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="51">
-        <f>IF(B8&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B8" s="52" t="n"/>
-      <c r="C8" s="51" t="n"/>
-      <c r="D8" s="53" t="n"/>
-      <c r="E8" s="52" t="n"/>
-      <c r="F8" s="51" t="n"/>
-      <c r="G8" s="53" t="n"/>
-      <c r="H8" s="52" t="n"/>
-      <c r="I8" s="51" t="n"/>
-      <c r="J8" s="51" t="n"/>
-      <c r="K8" s="53" t="n"/>
-      <c r="L8" s="53" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="51">
-        <f>IF(B9&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B9" s="52" t="n"/>
-      <c r="C9" s="51" t="n"/>
-      <c r="D9" s="53" t="n"/>
-      <c r="E9" s="52" t="n"/>
-      <c r="F9" s="51" t="n"/>
-      <c r="G9" s="53" t="n"/>
-      <c r="H9" s="52" t="n"/>
-      <c r="I9" s="51" t="n"/>
-      <c r="J9" s="51" t="n"/>
-      <c r="K9" s="53" t="n"/>
-      <c r="L9" s="53" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="51">
-        <f>IF(B10&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B10" s="52" t="n"/>
-      <c r="C10" s="51" t="n"/>
-      <c r="D10" s="53" t="n"/>
-      <c r="E10" s="52" t="n"/>
-      <c r="F10" s="51" t="n"/>
-      <c r="G10" s="53" t="n"/>
-      <c r="H10" s="52" t="n"/>
-      <c r="I10" s="51" t="n"/>
-      <c r="J10" s="51" t="n"/>
-      <c r="K10" s="53" t="n"/>
-      <c r="L10" s="53" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="51">
-        <f>IF(B11&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B11" s="52" t="n"/>
-      <c r="C11" s="51" t="n"/>
-      <c r="D11" s="53" t="n"/>
-      <c r="E11" s="52" t="n"/>
-      <c r="F11" s="51" t="n"/>
-      <c r="G11" s="53" t="n"/>
-      <c r="H11" s="52" t="n"/>
-      <c r="I11" s="51" t="n"/>
-      <c r="J11" s="51" t="n"/>
-      <c r="K11" s="53" t="n"/>
-      <c r="L11" s="53" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="51">
-        <f>IF(B12&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B12" s="52" t="n"/>
-      <c r="C12" s="51" t="n"/>
-      <c r="D12" s="53" t="n"/>
-      <c r="E12" s="52" t="n"/>
-      <c r="F12" s="51" t="n"/>
-      <c r="G12" s="53" t="n"/>
-      <c r="H12" s="52" t="n"/>
-      <c r="I12" s="51" t="n"/>
-      <c r="J12" s="51" t="n"/>
-      <c r="K12" s="53" t="n"/>
-      <c r="L12" s="53" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="51">
-        <f>IF(B13&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B13" s="52" t="n"/>
-      <c r="C13" s="51" t="n"/>
-      <c r="D13" s="53" t="n"/>
-      <c r="E13" s="52" t="n"/>
-      <c r="F13" s="51" t="n"/>
-      <c r="G13" s="53" t="n"/>
-      <c r="H13" s="52" t="n"/>
-      <c r="I13" s="51" t="n"/>
-      <c r="J13" s="51" t="n"/>
-      <c r="K13" s="53" t="n"/>
-      <c r="L13" s="53" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="51">
-        <f>IF(B14&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B14" s="52" t="n"/>
-      <c r="C14" s="51" t="n"/>
-      <c r="D14" s="53" t="n"/>
-      <c r="E14" s="52" t="n"/>
-      <c r="F14" s="51" t="n"/>
-      <c r="G14" s="53" t="n"/>
-      <c r="H14" s="52" t="n"/>
-      <c r="I14" s="51" t="n"/>
-      <c r="J14" s="51" t="n"/>
-      <c r="K14" s="53" t="n"/>
-      <c r="L14" s="53" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="51">
-        <f>IF(B15&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B15" s="52" t="n"/>
-      <c r="C15" s="51" t="n"/>
-      <c r="D15" s="53" t="n"/>
-      <c r="E15" s="52" t="n"/>
-      <c r="F15" s="51" t="n"/>
-      <c r="G15" s="53" t="n"/>
-      <c r="H15" s="52" t="n"/>
-      <c r="I15" s="51" t="n"/>
-      <c r="J15" s="51" t="n"/>
-      <c r="K15" s="53" t="n"/>
-      <c r="L15" s="53" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="51">
-        <f>IF(B16&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B16" s="52" t="n"/>
-      <c r="C16" s="51" t="n"/>
-      <c r="D16" s="53" t="n"/>
-      <c r="E16" s="52" t="n"/>
-      <c r="F16" s="51" t="n"/>
-      <c r="G16" s="53" t="n"/>
-      <c r="H16" s="52" t="n"/>
-      <c r="I16" s="51" t="n"/>
-      <c r="J16" s="51" t="n"/>
-      <c r="K16" s="53" t="n"/>
-      <c r="L16" s="53" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="51">
-        <f>IF(B17&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B17" s="52" t="n"/>
-      <c r="C17" s="51" t="n"/>
-      <c r="D17" s="53" t="n"/>
-      <c r="E17" s="52" t="n"/>
-      <c r="F17" s="51" t="n"/>
-      <c r="G17" s="53" t="n"/>
-      <c r="H17" s="52" t="n"/>
-      <c r="I17" s="51" t="n"/>
-      <c r="J17" s="51" t="n"/>
-      <c r="K17" s="53" t="n"/>
-      <c r="L17" s="53" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="51">
-        <f>IF(B18&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B18" s="52" t="n"/>
-      <c r="C18" s="51" t="n"/>
-      <c r="D18" s="53" t="n"/>
-      <c r="E18" s="52" t="n"/>
-      <c r="F18" s="51" t="n"/>
-      <c r="G18" s="53" t="n"/>
-      <c r="H18" s="52" t="n"/>
-      <c r="I18" s="51" t="n"/>
-      <c r="J18" s="51" t="n"/>
-      <c r="K18" s="53" t="n"/>
-      <c r="L18" s="53" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="51">
-        <f>IF(B19&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B19" s="52" t="n"/>
-      <c r="C19" s="51" t="n"/>
-      <c r="D19" s="53" t="n"/>
-      <c r="E19" s="52" t="n"/>
-      <c r="F19" s="51" t="n"/>
-      <c r="G19" s="53" t="n"/>
-      <c r="H19" s="52" t="n"/>
-      <c r="I19" s="51" t="n"/>
-      <c r="J19" s="51" t="n"/>
-      <c r="K19" s="53" t="n"/>
-      <c r="L19" s="53" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="51">
-        <f>IF(B20&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B20" s="52" t="n"/>
-      <c r="C20" s="51" t="n"/>
-      <c r="D20" s="53" t="n"/>
-      <c r="E20" s="52" t="n"/>
-      <c r="F20" s="51" t="n"/>
-      <c r="G20" s="53" t="n"/>
-      <c r="H20" s="52" t="n"/>
-      <c r="I20" s="51" t="n"/>
-      <c r="J20" s="51" t="n"/>
-      <c r="K20" s="53" t="n"/>
-      <c r="L20" s="53" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="51">
-        <f>IF(B21&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B21" s="52" t="n"/>
-      <c r="C21" s="51" t="n"/>
-      <c r="D21" s="53" t="n"/>
-      <c r="E21" s="52" t="n"/>
-      <c r="F21" s="51" t="n"/>
-      <c r="G21" s="53" t="n"/>
-      <c r="H21" s="52" t="n"/>
-      <c r="I21" s="51" t="n"/>
-      <c r="J21" s="51" t="n"/>
-      <c r="K21" s="53" t="n"/>
-      <c r="L21" s="53" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="51">
-        <f>IF(B22&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B22" s="52" t="n"/>
-      <c r="C22" s="51" t="n"/>
-      <c r="D22" s="53" t="n"/>
-      <c r="E22" s="52" t="n"/>
-      <c r="F22" s="51" t="n"/>
-      <c r="G22" s="53" t="n"/>
-      <c r="H22" s="52" t="n"/>
-      <c r="I22" s="51" t="n"/>
-      <c r="J22" s="51" t="n"/>
-      <c r="K22" s="53" t="n"/>
-      <c r="L22" s="53" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="51">
-        <f>IF(B23&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B23" s="52" t="n"/>
-      <c r="C23" s="51" t="n"/>
-      <c r="D23" s="53" t="n"/>
-      <c r="E23" s="52" t="n"/>
-      <c r="F23" s="51" t="n"/>
-      <c r="G23" s="53" t="n"/>
-      <c r="H23" s="52" t="n"/>
-      <c r="I23" s="51" t="n"/>
-      <c r="J23" s="51" t="n"/>
-      <c r="K23" s="53" t="n"/>
-      <c r="L23" s="53" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="51">
-        <f>IF(B24&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B24" s="52" t="n"/>
-      <c r="C24" s="51" t="n"/>
-      <c r="D24" s="53" t="n"/>
-      <c r="E24" s="52" t="n"/>
-      <c r="F24" s="51" t="n"/>
-      <c r="G24" s="53" t="n"/>
-      <c r="H24" s="52" t="n"/>
-      <c r="I24" s="51" t="n"/>
-      <c r="J24" s="51" t="n"/>
-      <c r="K24" s="53" t="n"/>
-      <c r="L24" s="53" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="51">
-        <f>IF(B25&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B25" s="52" t="n"/>
-      <c r="C25" s="51" t="n"/>
-      <c r="D25" s="53" t="n"/>
-      <c r="E25" s="52" t="n"/>
-      <c r="F25" s="51" t="n"/>
-      <c r="G25" s="53" t="n"/>
-      <c r="H25" s="52" t="n"/>
-      <c r="I25" s="51" t="n"/>
-      <c r="J25" s="51" t="n"/>
-      <c r="K25" s="53" t="n"/>
-      <c r="L25" s="53" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="51">
-        <f>IF(B26&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B26" s="52" t="n"/>
-      <c r="C26" s="51" t="n"/>
-      <c r="D26" s="53" t="n"/>
-      <c r="E26" s="52" t="n"/>
-      <c r="F26" s="51" t="n"/>
-      <c r="G26" s="53" t="n"/>
-      <c r="H26" s="52" t="n"/>
-      <c r="I26" s="51" t="n"/>
-      <c r="J26" s="51" t="n"/>
-      <c r="K26" s="53" t="n"/>
-      <c r="L26" s="53" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="51">
-        <f>IF(B27&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B27" s="52" t="n"/>
-      <c r="C27" s="51" t="n"/>
-      <c r="D27" s="53" t="n"/>
-      <c r="E27" s="52" t="n"/>
-      <c r="F27" s="51" t="n"/>
-      <c r="G27" s="53" t="n"/>
-      <c r="H27" s="52" t="n"/>
-      <c r="I27" s="51" t="n"/>
-      <c r="J27" s="51" t="n"/>
-      <c r="K27" s="53" t="n"/>
-      <c r="L27" s="53" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="51">
-        <f>IF(B28&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B28" s="52" t="n"/>
-      <c r="C28" s="51" t="n"/>
-      <c r="D28" s="53" t="n"/>
-      <c r="E28" s="52" t="n"/>
-      <c r="F28" s="51" t="n"/>
-      <c r="G28" s="53" t="n"/>
-      <c r="H28" s="52" t="n"/>
-      <c r="I28" s="51" t="n"/>
-      <c r="J28" s="51" t="n"/>
-      <c r="K28" s="53" t="n"/>
-      <c r="L28" s="53" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="51">
-        <f>IF(B29&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B29" s="52" t="n"/>
-      <c r="C29" s="51" t="n"/>
-      <c r="D29" s="53" t="n"/>
-      <c r="E29" s="52" t="n"/>
-      <c r="F29" s="51" t="n"/>
-      <c r="G29" s="53" t="n"/>
-      <c r="H29" s="52" t="n"/>
-      <c r="I29" s="51" t="n"/>
-      <c r="J29" s="51" t="n"/>
-      <c r="K29" s="53" t="n"/>
-      <c r="L29" s="53" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="51">
-        <f>IF(B30&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B30" s="52" t="n"/>
-      <c r="C30" s="51" t="n"/>
-      <c r="D30" s="53" t="n"/>
-      <c r="E30" s="52" t="n"/>
-      <c r="F30" s="51" t="n"/>
-      <c r="G30" s="53" t="n"/>
-      <c r="H30" s="52" t="n"/>
-      <c r="I30" s="51" t="n"/>
-      <c r="J30" s="51" t="n"/>
-      <c r="K30" s="53" t="n"/>
-      <c r="L30" s="53" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="51">
-        <f>IF(B31&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B31" s="52" t="n"/>
-      <c r="C31" s="51" t="n"/>
-      <c r="D31" s="53" t="n"/>
-      <c r="E31" s="52" t="n"/>
-      <c r="F31" s="51" t="n"/>
-      <c r="G31" s="53" t="n"/>
-      <c r="H31" s="52" t="n"/>
-      <c r="I31" s="51" t="n"/>
-      <c r="J31" s="51" t="n"/>
-      <c r="K31" s="53" t="n"/>
-      <c r="L31" s="53" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="51">
-        <f>IF(B32&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B32" s="52" t="n"/>
-      <c r="C32" s="51" t="n"/>
-      <c r="D32" s="53" t="n"/>
-      <c r="E32" s="52" t="n"/>
-      <c r="F32" s="51" t="n"/>
-      <c r="G32" s="53" t="n"/>
-      <c r="H32" s="52" t="n"/>
-      <c r="I32" s="51" t="n"/>
-      <c r="J32" s="51" t="n"/>
-      <c r="K32" s="53" t="n"/>
-      <c r="L32" s="53" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="51">
-        <f>IF(B33&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B33" s="52" t="n"/>
-      <c r="C33" s="51" t="n"/>
-      <c r="D33" s="53" t="n"/>
-      <c r="E33" s="52" t="n"/>
-      <c r="F33" s="51" t="n"/>
-      <c r="G33" s="53" t="n"/>
-      <c r="H33" s="52" t="n"/>
-      <c r="I33" s="51" t="n"/>
-      <c r="J33" s="51" t="n"/>
-      <c r="K33" s="53" t="n"/>
-      <c r="L33" s="53" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="51">
-        <f>IF(B34&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B34" s="52" t="n"/>
-      <c r="C34" s="51" t="n"/>
-      <c r="D34" s="53" t="n"/>
-      <c r="E34" s="52" t="n"/>
-      <c r="F34" s="51" t="n"/>
-      <c r="G34" s="53" t="n"/>
-      <c r="H34" s="52" t="n"/>
-      <c r="I34" s="51" t="n"/>
-      <c r="J34" s="51" t="n"/>
-      <c r="K34" s="53" t="n"/>
-      <c r="L34" s="53" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="51">
-        <f>IF(B35&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B35" s="52" t="n"/>
-      <c r="C35" s="51" t="n"/>
-      <c r="D35" s="53" t="n"/>
-      <c r="E35" s="52" t="n"/>
-      <c r="F35" s="51" t="n"/>
-      <c r="G35" s="53" t="n"/>
-      <c r="H35" s="52" t="n"/>
-      <c r="I35" s="51" t="n"/>
-      <c r="J35" s="51" t="n"/>
-      <c r="K35" s="53" t="n"/>
-      <c r="L35" s="53" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="51">
-        <f>IF(B36&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B36" s="52" t="n"/>
-      <c r="C36" s="51" t="n"/>
-      <c r="D36" s="53" t="n"/>
-      <c r="E36" s="52" t="n"/>
-      <c r="F36" s="51" t="n"/>
-      <c r="G36" s="53" t="n"/>
-      <c r="H36" s="52" t="n"/>
-      <c r="I36" s="51" t="n"/>
-      <c r="J36" s="51" t="n"/>
-      <c r="K36" s="53" t="n"/>
-      <c r="L36" s="53" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="51">
-        <f>IF(B37&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B37" s="52" t="n"/>
-      <c r="C37" s="51" t="n"/>
-      <c r="D37" s="53" t="n"/>
-      <c r="E37" s="52" t="n"/>
-      <c r="F37" s="51" t="n"/>
-      <c r="G37" s="53" t="n"/>
-      <c r="H37" s="52" t="n"/>
-      <c r="I37" s="51" t="n"/>
-      <c r="J37" s="51" t="n"/>
-      <c r="K37" s="53" t="n"/>
-      <c r="L37" s="53" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="51">
-        <f>IF(B38&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B38" s="52" t="n"/>
-      <c r="C38" s="51" t="n"/>
-      <c r="D38" s="53" t="n"/>
-      <c r="E38" s="52" t="n"/>
-      <c r="F38" s="51" t="n"/>
-      <c r="G38" s="53" t="n"/>
-      <c r="H38" s="52" t="n"/>
-      <c r="I38" s="51" t="n"/>
-      <c r="J38" s="51" t="n"/>
-      <c r="K38" s="53" t="n"/>
-      <c r="L38" s="53" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="51">
-        <f>IF(B39&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B39" s="52" t="n"/>
-      <c r="C39" s="51" t="n"/>
-      <c r="D39" s="53" t="n"/>
-      <c r="E39" s="52" t="n"/>
-      <c r="F39" s="51" t="n"/>
-      <c r="G39" s="53" t="n"/>
-      <c r="H39" s="52" t="n"/>
-      <c r="I39" s="51" t="n"/>
-      <c r="J39" s="51" t="n"/>
-      <c r="K39" s="53" t="n"/>
-      <c r="L39" s="53" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="51">
-        <f>IF(B40&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B40" s="52" t="n"/>
-      <c r="C40" s="51" t="n"/>
-      <c r="D40" s="53" t="n"/>
-      <c r="E40" s="52" t="n"/>
-      <c r="F40" s="51" t="n"/>
-      <c r="G40" s="53" t="n"/>
-      <c r="H40" s="52" t="n"/>
-      <c r="I40" s="51" t="n"/>
-      <c r="J40" s="51" t="n"/>
-      <c r="K40" s="53" t="n"/>
-      <c r="L40" s="53" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="51">
-        <f>IF(B41&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B41" s="52" t="n"/>
-      <c r="C41" s="51" t="n"/>
-      <c r="D41" s="53" t="n"/>
-      <c r="E41" s="52" t="n"/>
-      <c r="F41" s="51" t="n"/>
-      <c r="G41" s="53" t="n"/>
-      <c r="H41" s="52" t="n"/>
-      <c r="I41" s="51" t="n"/>
-      <c r="J41" s="51" t="n"/>
-      <c r="K41" s="53" t="n"/>
-      <c r="L41" s="53" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="51">
-        <f>IF(B42&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B42" s="52" t="n"/>
-      <c r="C42" s="51" t="n"/>
-      <c r="D42" s="53" t="n"/>
-      <c r="E42" s="52" t="n"/>
-      <c r="F42" s="51" t="n"/>
-      <c r="G42" s="53" t="n"/>
-      <c r="H42" s="52" t="n"/>
-      <c r="I42" s="51" t="n"/>
-      <c r="J42" s="51" t="n"/>
-      <c r="K42" s="53" t="n"/>
-      <c r="L42" s="53" t="n"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="51">
-        <f>IF(B43&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B43" s="52" t="n"/>
-      <c r="C43" s="51" t="n"/>
-      <c r="D43" s="53" t="n"/>
-      <c r="E43" s="52" t="n"/>
-      <c r="F43" s="51" t="n"/>
-      <c r="G43" s="53" t="n"/>
-      <c r="H43" s="52" t="n"/>
-      <c r="I43" s="51" t="n"/>
-      <c r="J43" s="51" t="n"/>
-      <c r="K43" s="53" t="n"/>
-      <c r="L43" s="53" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="51">
-        <f>IF(B44&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B44" s="52" t="n"/>
-      <c r="C44" s="51" t="n"/>
-      <c r="D44" s="53" t="n"/>
-      <c r="E44" s="52" t="n"/>
-      <c r="F44" s="51" t="n"/>
-      <c r="G44" s="53" t="n"/>
-      <c r="H44" s="52" t="n"/>
-      <c r="I44" s="51" t="n"/>
-      <c r="J44" s="51" t="n"/>
-      <c r="K44" s="53" t="n"/>
-      <c r="L44" s="53" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="51">
-        <f>IF(B45&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B45" s="52" t="n"/>
-      <c r="C45" s="51" t="n"/>
-      <c r="D45" s="53" t="n"/>
-      <c r="E45" s="52" t="n"/>
-      <c r="F45" s="51" t="n"/>
-      <c r="G45" s="53" t="n"/>
-      <c r="H45" s="52" t="n"/>
-      <c r="I45" s="51" t="n"/>
-      <c r="J45" s="51" t="n"/>
-      <c r="K45" s="53" t="n"/>
-      <c r="L45" s="53" t="n"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="51">
-        <f>IF(B46&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B46" s="52" t="n"/>
-      <c r="C46" s="51" t="n"/>
-      <c r="D46" s="53" t="n"/>
-      <c r="E46" s="52" t="n"/>
-      <c r="F46" s="51" t="n"/>
-      <c r="G46" s="53" t="n"/>
-      <c r="H46" s="52" t="n"/>
-      <c r="I46" s="51" t="n"/>
-      <c r="J46" s="51" t="n"/>
-      <c r="K46" s="53" t="n"/>
-      <c r="L46" s="53" t="n"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="51">
-        <f>IF(B47&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B47" s="52" t="n"/>
-      <c r="C47" s="51" t="n"/>
-      <c r="D47" s="53" t="n"/>
-      <c r="E47" s="52" t="n"/>
-      <c r="F47" s="51" t="n"/>
-      <c r="G47" s="53" t="n"/>
-      <c r="H47" s="52" t="n"/>
-      <c r="I47" s="51" t="n"/>
-      <c r="J47" s="51" t="n"/>
-      <c r="K47" s="53" t="n"/>
-      <c r="L47" s="53" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="51">
-        <f>IF(B48&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B48" s="52" t="n"/>
-      <c r="C48" s="51" t="n"/>
-      <c r="D48" s="53" t="n"/>
-      <c r="E48" s="52" t="n"/>
-      <c r="F48" s="51" t="n"/>
-      <c r="G48" s="53" t="n"/>
-      <c r="H48" s="52" t="n"/>
-      <c r="I48" s="51" t="n"/>
-      <c r="J48" s="51" t="n"/>
-      <c r="K48" s="53" t="n"/>
-      <c r="L48" s="53" t="n"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="51">
-        <f>IF(B49&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B49" s="52" t="n"/>
-      <c r="C49" s="51" t="n"/>
-      <c r="D49" s="53" t="n"/>
-      <c r="E49" s="52" t="n"/>
-      <c r="F49" s="51" t="n"/>
-      <c r="G49" s="53" t="n"/>
-      <c r="H49" s="52" t="n"/>
-      <c r="I49" s="51" t="n"/>
-      <c r="J49" s="51" t="n"/>
-      <c r="K49" s="53" t="n"/>
-      <c r="L49" s="53" t="n"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="51">
-        <f>IF(B50&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B50" s="52" t="n"/>
-      <c r="C50" s="51" t="n"/>
-      <c r="D50" s="53" t="n"/>
-      <c r="E50" s="52" t="n"/>
-      <c r="F50" s="51" t="n"/>
-      <c r="G50" s="53" t="n"/>
-      <c r="H50" s="52" t="n"/>
-      <c r="I50" s="51" t="n"/>
-      <c r="J50" s="51" t="n"/>
-      <c r="K50" s="53" t="n"/>
-      <c r="L50" s="53" t="n"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="51">
-        <f>IF(B51&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B51" s="52" t="n"/>
-      <c r="C51" s="51" t="n"/>
-      <c r="D51" s="53" t="n"/>
-      <c r="E51" s="52" t="n"/>
-      <c r="F51" s="51" t="n"/>
-      <c r="G51" s="53" t="n"/>
-      <c r="H51" s="52" t="n"/>
-      <c r="I51" s="51" t="n"/>
-      <c r="J51" s="51" t="n"/>
-      <c r="K51" s="53" t="n"/>
-      <c r="L51" s="53" t="n"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="51">
-        <f>IF(B52&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B52" s="52" t="n"/>
-      <c r="C52" s="51" t="n"/>
-      <c r="D52" s="53" t="n"/>
-      <c r="E52" s="52" t="n"/>
-      <c r="F52" s="51" t="n"/>
-      <c r="G52" s="53" t="n"/>
-      <c r="H52" s="52" t="n"/>
-      <c r="I52" s="51" t="n"/>
-      <c r="J52" s="51" t="n"/>
-      <c r="K52" s="53" t="n"/>
-      <c r="L52" s="53" t="n"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="51">
-        <f>IF(B53&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B53" s="52" t="n"/>
-      <c r="C53" s="51" t="n"/>
-      <c r="D53" s="53" t="n"/>
-      <c r="E53" s="52" t="n"/>
-      <c r="F53" s="51" t="n"/>
-      <c r="G53" s="53" t="n"/>
-      <c r="H53" s="52" t="n"/>
-      <c r="I53" s="51" t="n"/>
-      <c r="J53" s="51" t="n"/>
-      <c r="K53" s="53" t="n"/>
-      <c r="L53" s="53" t="n"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="51">
-        <f>IF(B54&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B54" s="52" t="n"/>
-      <c r="C54" s="51" t="n"/>
-      <c r="D54" s="53" t="n"/>
-      <c r="E54" s="52" t="n"/>
-      <c r="F54" s="51" t="n"/>
-      <c r="G54" s="53" t="n"/>
-      <c r="H54" s="52" t="n"/>
-      <c r="I54" s="51" t="n"/>
-      <c r="J54" s="51" t="n"/>
-      <c r="K54" s="53" t="n"/>
-      <c r="L54" s="53" t="n"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="51">
-        <f>IF(B55&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="52" t="n"/>
-      <c r="C55" s="51" t="n"/>
-      <c r="D55" s="53" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="51" t="n"/>
-      <c r="J55" s="51" t="n"/>
-      <c r="K55" s="53" t="n"/>
-      <c r="L55" s="53" t="n"/>
-    </row>
-  </sheetData>
-  <autoFilter ref="A4:L55"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
@@ -4888,7 +3752,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00DC3545"/>
@@ -4927,88 +3791,88 @@
       </c>
     </row>
     <row r="2" ht="60" customHeight="1">
-      <c r="A2" s="55" t="inlineStr">
+      <c r="A2" s="54" t="inlineStr">
         <is>
           <t>D</t>
         </is>
       </c>
-      <c r="B2" s="56" t="inlineStr">
+      <c r="B2" s="55" t="inlineStr">
         <is>
           <t>Fehler mit gravierenden Folgen</t>
         </is>
       </c>
-      <c r="C2" s="57" t="inlineStr">
+      <c r="C2" s="56" t="inlineStr">
         <is>
           <t>daraus resultierende schwere Gesundheitsschäden, wesentliche finanzielle Nachteile oder ein erheblicher Imageverlust</t>
         </is>
       </c>
-      <c r="D2" s="57" t="inlineStr">
+      <c r="D2" s="56" t="inlineStr">
         <is>
           <t>gesetzl. vorgeschriebene Unterweisungen oder Überprüfungen liegen nicht vor, Behandlungsfehler mit Konsequenzen, Defekte von Notfallgeräten</t>
         </is>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
-      <c r="A3" s="58" t="inlineStr">
+      <c r="A3" s="57" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B3" s="59" t="inlineStr">
+      <c r="B3" s="58" t="inlineStr">
         <is>
           <t>Fehler mit leichten bis mittelschweren Folgen</t>
         </is>
       </c>
-      <c r="C3" s="60" t="inlineStr">
+      <c r="C3" s="59" t="inlineStr">
         <is>
           <t>Fehler mit Gesundheitsschäden, Einsatzfähigkeit HSM gefährdet, Fehler führte zu externer Kundenbeschwerde, Vorgegebener Standard wird nicht durchgeführt</t>
         </is>
       </c>
-      <c r="D3" s="60" t="inlineStr">
+      <c r="D3" s="59" t="inlineStr">
         <is>
           <t>Behandlungsfehler ohne Konsequenzen, Termin- oder Materialkonflikt nicht rechtzeitig erkannt, Ausgang von Medikamenten, NADOK Protokolle nicht vollständig ausgefüllt</t>
         </is>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
-      <c r="A4" s="61" t="inlineStr">
+      <c r="A4" s="60" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="B4" s="62" t="inlineStr">
+      <c r="B4" s="61" t="inlineStr">
         <is>
           <t>Beinahefehler ohne Folgen</t>
         </is>
       </c>
-      <c r="C4" s="63" t="inlineStr">
+      <c r="C4" s="62" t="inlineStr">
         <is>
           <t>ein Fehler wurde noch vor seinem wirksamen Eintreten erkannt, bzw. durch Gegenmaßnahmen können Folgen noch abgefangen werden</t>
         </is>
       </c>
-      <c r="D4" s="63" t="inlineStr">
+      <c r="D4" s="62" t="inlineStr">
         <is>
           <t>Termin- oder Materialkonflikt gerade noch rechtzeitig erkannt und behoben</t>
         </is>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
-      <c r="A5" s="64" t="inlineStr">
+      <c r="A5" s="63" t="inlineStr">
         <is>
           <t>A</t>
         </is>
       </c>
-      <c r="B5" s="65" t="inlineStr">
+      <c r="B5" s="64" t="inlineStr">
         <is>
           <t>unsichere Handlung</t>
         </is>
       </c>
-      <c r="C5" s="66" t="inlineStr">
+      <c r="C5" s="65" t="inlineStr">
         <is>
           <t>es wird unsauber gearbeitet, aber es entsteht kein Schaden</t>
         </is>
       </c>
-      <c r="D5" s="66" t="inlineStr">
+      <c r="D5" s="65" t="inlineStr">
         <is>
           <t>Vorgaben werden nicht eingehalten, z.B. Eintrag der RTW Checks in FB 260</t>
         </is>
@@ -5019,14 +3883,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00666666"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5068,296 +3932,300 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="67" t="inlineStr">
+      <c r="A3" s="66" t="inlineStr">
         <is>
           <t>Dr. Markus Frei</t>
         </is>
       </c>
-      <c r="B3" s="67" t="inlineStr">
+      <c r="B3" s="66" t="inlineStr">
         <is>
           <t>markus.frei@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C3" s="68" t="inlineStr">
-        <is>
-          <t>Arzt / Leiter Getriebewerk</t>
-        </is>
-      </c>
-      <c r="D3" s="67" t="inlineStr"/>
+      <c r="C3" s="67" t="inlineStr">
+        <is>
+          <t>Arzt</t>
+        </is>
+      </c>
+      <c r="D3" s="66" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="69" t="inlineStr">
+      <c r="A4" s="68" t="inlineStr">
         <is>
           <t>Dr. Sabine Schmidt</t>
         </is>
       </c>
-      <c r="B4" s="69" t="inlineStr">
+      <c r="B4" s="68" t="inlineStr">
         <is>
           <t>sabine.m.schmidt@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C4" s="70" t="inlineStr">
+      <c r="C4" s="69" t="inlineStr">
         <is>
           <t>Ärztin</t>
         </is>
       </c>
-      <c r="D4" s="69" t="inlineStr"/>
+      <c r="D4" s="68" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="67" t="inlineStr">
+      <c r="A5" s="66" t="inlineStr">
         <is>
           <t>Dr. Lilla Vitez</t>
         </is>
       </c>
-      <c r="B5" s="67" t="inlineStr">
+      <c r="B5" s="66" t="inlineStr">
         <is>
           <t>lilla.vitez@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C5" s="68" t="inlineStr">
+      <c r="C5" s="67" t="inlineStr">
         <is>
           <t>Ärztin</t>
         </is>
       </c>
-      <c r="D5" s="67" t="inlineStr"/>
+      <c r="D5" s="66" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="69" t="inlineStr">
+      <c r="A6" s="68" t="inlineStr">
         <is>
           <t>Bernd Breig</t>
         </is>
       </c>
-      <c r="B6" s="69" t="inlineStr">
+      <c r="B6" s="68" t="inlineStr">
         <is>
           <t>bernd.breig@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C6" s="70" t="inlineStr">
+      <c r="C6" s="69" t="inlineStr">
         <is>
           <t>Stv. Med.&amp;Verbr.-stoff</t>
         </is>
       </c>
-      <c r="D6" s="69" t="inlineStr"/>
+      <c r="D6" s="68" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="67" t="inlineStr">
+      <c r="A7" s="66" t="inlineStr">
         <is>
           <t>Elke Krempl</t>
         </is>
       </c>
-      <c r="B7" s="67" t="inlineStr">
+      <c r="B7" s="66" t="inlineStr">
         <is>
           <t>elke.krempl@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C7" s="68" t="inlineStr">
+      <c r="C7" s="67" t="inlineStr">
         <is>
           <t>Mitarbeiterin</t>
         </is>
       </c>
-      <c r="D7" s="67" t="inlineStr"/>
+      <c r="D7" s="66" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="69" t="inlineStr">
+      <c r="A8" s="68" t="inlineStr">
         <is>
           <t>Emanuel Siebert</t>
         </is>
       </c>
-      <c r="B8" s="69" t="inlineStr">
+      <c r="B8" s="68" t="inlineStr">
         <is>
           <t>emanuel.siebert@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C8" s="70" t="inlineStr">
+      <c r="C8" s="69" t="inlineStr">
         <is>
           <t>Leiter EDV</t>
         </is>
       </c>
-      <c r="D8" s="69" t="inlineStr"/>
+      <c r="D8" s="68" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="67" t="inlineStr">
+      <c r="A9" s="66" t="inlineStr">
         <is>
           <t>Walter Putschler</t>
         </is>
       </c>
-      <c r="B9" s="67" t="inlineStr">
+      <c r="B9" s="66" t="inlineStr">
         <is>
           <t>walter.putschler@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C9" s="68" t="inlineStr">
+      <c r="C9" s="67" t="inlineStr">
         <is>
           <t>Leiter Ablauf&amp;Prozessprobleme</t>
         </is>
       </c>
-      <c r="D9" s="67" t="inlineStr">
+      <c r="D9" s="66" t="inlineStr">
         <is>
           <t>BCC-Empfänger</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="69" t="inlineStr">
+      <c r="A10" s="68" t="inlineStr">
         <is>
           <t>Benjamin Jochim</t>
         </is>
       </c>
-      <c r="B10" s="69" t="inlineStr">
+      <c r="B10" s="68" t="inlineStr">
         <is>
           <t>benjamin.jochim@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C10" s="70" t="inlineStr">
+      <c r="C10" s="69" t="inlineStr">
         <is>
           <t>Mitarbeiter</t>
         </is>
       </c>
-      <c r="D10" s="69" t="inlineStr"/>
+      <c r="D10" s="68" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="67" t="inlineStr">
+      <c r="A11" s="66" t="inlineStr">
         <is>
           <t>Harry Zuber</t>
         </is>
       </c>
-      <c r="B11" s="67" t="inlineStr">
+      <c r="B11" s="66" t="inlineStr">
         <is>
           <t>harry.zuber@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C11" s="68" t="inlineStr">
+      <c r="C11" s="67" t="inlineStr">
         <is>
           <t>Mitarbeiter</t>
         </is>
       </c>
-      <c r="D11" s="67" t="inlineStr"/>
+      <c r="D11" s="66" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="69" t="inlineStr">
+      <c r="A12" s="68" t="inlineStr">
         <is>
           <t>Markus Göpfrich</t>
         </is>
       </c>
-      <c r="B12" s="69" t="inlineStr">
+      <c r="B12" s="68" t="inlineStr">
         <is>
           <t>Markus.Goepfrich@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C12" s="70" t="inlineStr">
+      <c r="C12" s="69" t="inlineStr">
         <is>
           <t>Leiter RTW &amp; MPG</t>
         </is>
       </c>
-      <c r="D12" s="69" t="inlineStr"/>
+      <c r="D12" s="68" t="inlineStr">
+        <is>
+          <t>Name im Dropdown: Göpfrich</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="67" t="inlineStr">
+      <c r="A13" s="66" t="inlineStr">
         <is>
           <t>Tobias Zeller</t>
         </is>
       </c>
-      <c r="B13" s="67" t="inlineStr">
+      <c r="B13" s="66" t="inlineStr">
         <is>
           <t>tobias_felix.zeller@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C13" s="68" t="inlineStr">
+      <c r="C13" s="67" t="inlineStr">
         <is>
           <t>Leiter Med.&amp;Verbr.-stoff</t>
         </is>
       </c>
-      <c r="D13" s="67" t="inlineStr"/>
+      <c r="D13" s="66" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="69" t="inlineStr">
+      <c r="A14" s="68" t="inlineStr">
         <is>
           <t>Emily Kim Schmidt</t>
         </is>
       </c>
-      <c r="B14" s="69" t="inlineStr">
+      <c r="B14" s="68" t="inlineStr">
         <is>
           <t>emily_kim.schmidt@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C14" s="70" t="inlineStr">
+      <c r="C14" s="69" t="inlineStr">
         <is>
           <t>Leiterin Sekretariat</t>
         </is>
       </c>
-      <c r="D14" s="69" t="inlineStr"/>
+      <c r="D14" s="68" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="67" t="inlineStr">
+      <c r="A15" s="66" t="inlineStr">
         <is>
           <t>Katrin Zieger-Buchta</t>
         </is>
       </c>
-      <c r="B15" s="67" t="inlineStr">
+      <c r="B15" s="66" t="inlineStr">
         <is>
           <t>katrin.zieger-buchta@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C15" s="68" t="inlineStr">
+      <c r="C15" s="67" t="inlineStr">
         <is>
           <t>Leiterin BGF</t>
         </is>
       </c>
-      <c r="D15" s="67" t="inlineStr"/>
+      <c r="D15" s="66" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="69" t="inlineStr">
+      <c r="A16" s="68" t="inlineStr">
         <is>
           <t>Susanne Müller-Horn</t>
         </is>
       </c>
-      <c r="B16" s="69" t="inlineStr">
+      <c r="B16" s="68" t="inlineStr">
         <is>
           <t>Susanne.Mueller-Horn@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C16" s="70" t="inlineStr">
+      <c r="C16" s="69" t="inlineStr">
         <is>
           <t>Stv. BGF</t>
         </is>
       </c>
-      <c r="D16" s="69" t="inlineStr"/>
+      <c r="D16" s="68" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="67" t="inlineStr">
+      <c r="A17" s="66" t="inlineStr">
         <is>
           <t>Larissa Radimersky</t>
         </is>
       </c>
-      <c r="B17" s="67" t="inlineStr">
+      <c r="B17" s="66" t="inlineStr">
         <is>
           <t>larissa.radimersky@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C17" s="68" t="inlineStr">
+      <c r="C17" s="67" t="inlineStr">
         <is>
           <t>Stv. Sekretariat</t>
         </is>
       </c>
-      <c r="D17" s="67" t="inlineStr"/>
+      <c r="D17" s="66" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="69" t="inlineStr">
+      <c r="A18" s="68" t="inlineStr">
         <is>
           <t>Fabian Wunsch</t>
         </is>
       </c>
-      <c r="B18" s="69" t="inlineStr">
+      <c r="B18" s="68" t="inlineStr">
         <is>
           <t>Fabian.Wunsch@mercedes-benz.com</t>
         </is>
       </c>
-      <c r="C18" s="70" t="inlineStr">
+      <c r="C18" s="69" t="inlineStr">
         <is>
           <t>Leiter WD-Fzg, Org. Ambulanz, Hygiene</t>
         </is>
       </c>
-      <c r="D18" s="69" t="inlineStr"/>
+      <c r="D18" s="68" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="F22" s="38" t="inlineStr">
@@ -5447,7 +4315,7 @@
     <row r="27">
       <c r="F27" s="37" t="inlineStr">
         <is>
-          <t>Goepfrich</t>
+          <t>Göpfrich</t>
         </is>
       </c>
       <c r="H27" s="37" t="inlineStr">
@@ -5459,7 +4327,7 @@
     <row r="28">
       <c r="F28" s="37" t="inlineStr">
         <is>
-          <t>Göpfrich</t>
+          <t>Jochim</t>
         </is>
       </c>
       <c r="H28" s="37" t="inlineStr">
@@ -5471,7 +4339,7 @@
     <row r="29">
       <c r="F29" s="37" t="inlineStr">
         <is>
-          <t>Jochim</t>
+          <t>Krempl</t>
         </is>
       </c>
       <c r="H29" s="37" t="inlineStr">
@@ -5483,7 +4351,7 @@
     <row r="30">
       <c r="F30" s="37" t="inlineStr">
         <is>
-          <t>Krempl</t>
+          <t>Müller-Horn</t>
         </is>
       </c>
       <c r="H30" s="37" t="inlineStr">
@@ -5495,7 +4363,7 @@
     <row r="31">
       <c r="F31" s="37" t="inlineStr">
         <is>
-          <t>Müller-Horn</t>
+          <t>Putschler</t>
         </is>
       </c>
       <c r="H31" s="37" t="inlineStr">
@@ -5507,7 +4375,7 @@
     <row r="32">
       <c r="F32" s="37" t="inlineStr">
         <is>
-          <t>Putschler</t>
+          <t>Radimersky</t>
         </is>
       </c>
       <c r="H32" s="37" t="inlineStr">
@@ -5519,7 +4387,7 @@
     <row r="33">
       <c r="F33" s="37" t="inlineStr">
         <is>
-          <t>Radimersky</t>
+          <t>Schmidt</t>
         </is>
       </c>
       <c r="H33" s="37" t="inlineStr">
@@ -5531,7 +4399,7 @@
     <row r="34">
       <c r="F34" s="37" t="inlineStr">
         <is>
-          <t>Schmidt</t>
+          <t>Siebert</t>
         </is>
       </c>
       <c r="H34" s="37" t="inlineStr">
@@ -5543,65 +4411,74 @@
     <row r="35">
       <c r="F35" s="37" t="inlineStr">
         <is>
-          <t>Siebert</t>
+          <t>Wunsch</t>
         </is>
       </c>
       <c r="H35" s="37" t="inlineStr">
         <is>
-          <t>Besprochen mit  Zeller</t>
+          <t>Besprochen mit  Jochim</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="F36" s="37" t="inlineStr">
         <is>
-          <t>Wunsch</t>
+          <t>Zeller</t>
         </is>
       </c>
       <c r="H36" s="37" t="inlineStr">
         <is>
-          <t>Besprochen mit  Schmidt</t>
+          <t>Besprochen mit  Wunsch</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="F37" s="37" t="inlineStr">
         <is>
-          <t>Zeller</t>
+          <t>Zieger-Buchta</t>
         </is>
       </c>
       <c r="H37" s="37" t="inlineStr">
         <is>
-          <t>Besprochen mit  Zieger-Buchta</t>
+          <t>Besprochen mit  Zeller</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="F38" s="37" t="inlineStr">
         <is>
-          <t>Zieger-Buchta</t>
+          <t>Zuber</t>
         </is>
       </c>
       <c r="H38" s="37" t="inlineStr">
         <is>
-          <t>Besprochen mit  Müller-Horn</t>
+          <t>Besprochen mit  Schmidt</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="F39" s="37" t="inlineStr">
-        <is>
-          <t>Zuber</t>
-        </is>
-      </c>
       <c r="H39" s="37" t="inlineStr">
         <is>
-          <t>Besprochen mit  Radimersky</t>
+          <t>Besprochen mit  Zieger-Buchta</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="H40" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Müller-Horn</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="H41" s="37" t="inlineStr">
+        <is>
+          <t>Besprochen mit  Radimersky</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="H42" s="37" t="inlineStr">
         <is>
           <t>Besprochen mit  Wunsch</t>
         </is>
@@ -5622,7 +4499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G51"/>
+  <dimension ref="B1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -6073,7 +4950,7 @@
       </c>
       <c r="D46" s="25" t="inlineStr">
         <is>
-          <t>Goepfrich</t>
+          <t>Göpfrich</t>
         </is>
       </c>
       <c r="F46" s="25" t="inlineStr"/>
@@ -6124,35 +5001,18 @@
     <row r="50">
       <c r="B50" s="25" t="inlineStr">
         <is>
-          <t>Getriebewerk</t>
+          <t>Hygiene</t>
         </is>
       </c>
       <c r="D50" s="25" t="inlineStr">
         <is>
-          <t>Dr.Frei</t>
-        </is>
-      </c>
-      <c r="F50" s="25" t="inlineStr">
-        <is>
-          <t>Dr.Schmidt</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="25" t="inlineStr">
-        <is>
-          <t>Hygiene</t>
-        </is>
-      </c>
-      <c r="D51" s="25" t="inlineStr">
-        <is>
           <t>Wunsch</t>
         </is>
       </c>
-      <c r="F51" s="25" t="inlineStr"/>
+      <c r="F50" s="25" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="55">
+  <mergeCells count="53">
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B47:C47"/>
     <mergeCell ref="C17:F17"/>
@@ -6201,8 +5061,6 @@
     <mergeCell ref="C31:F31"/>
     <mergeCell ref="B6:F6"/>
     <mergeCell ref="D42:E42"/>
-    <mergeCell ref="B51:C51"/>
-    <mergeCell ref="D51:E51"/>
     <mergeCell ref="B45:C45"/>
     <mergeCell ref="B50:C50"/>
     <mergeCell ref="C27:F27"/>
@@ -7277,7 +6135,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7412,141 +6270,56 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="52" t="n">
-        <v>45883.66136574074</v>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Frei</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>Laris geht nicht richtig und Meldeliste muss aktualisiert werden und Mailbutton geht nicht und es zeigt die Meldung der Active-X Inhalt ist blockiert</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="n">
-        <v>45884.45383101852</v>
-      </c>
-      <c r="F5" s="51" t="inlineStr">
-        <is>
-          <t>Zuber</t>
-        </is>
-      </c>
-      <c r="G5" s="53" t="inlineStr">
-        <is>
-          <t>Laris war nie kaputt, die Excel Anwendung muss für die Benutzung eingestellt werden im Bereich Active-X Inhalte</t>
-        </is>
-      </c>
-      <c r="H5" s="52" t="n">
-        <v>45884.45396990741</v>
-      </c>
-      <c r="I5" s="51" t="inlineStr">
-        <is>
-          <t>Zuber</t>
-        </is>
-      </c>
-      <c r="J5" s="54" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="K5" s="53" t="inlineStr"/>
-      <c r="L5" s="53" t="inlineStr">
-        <is>
-          <t>Nicht erforderlich</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="52" t="n">
-        <v>45926.35149305555</v>
-      </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Frei</t>
-        </is>
-      </c>
-      <c r="D6" s="53" t="inlineStr">
-        <is>
-          <t>Das Blatt Organisation Ambulanz in Laris hat einen Schreibschutz, so dass nichts eingetragen werden kann - bitte diesen entfernen</t>
-        </is>
-      </c>
-      <c r="E6" s="52" t="n">
-        <v>45926.45972222222</v>
-      </c>
-      <c r="F6" s="51" t="inlineStr">
-        <is>
-          <t>Siebert</t>
-        </is>
-      </c>
-      <c r="G6" s="53" t="inlineStr">
-        <is>
-          <t>Rechtsklick auf die Kachel -&gt; Schutz Pausieren</t>
-        </is>
-      </c>
-      <c r="H6" s="52" t="n">
-        <v>45926.45972222222</v>
-      </c>
-      <c r="I6" s="51" t="inlineStr">
-        <is>
-          <t>Siebert</t>
-        </is>
-      </c>
-      <c r="J6" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K6" s="53" t="inlineStr"/>
-      <c r="L6" s="53" t="inlineStr">
-        <is>
-          <t>REKO</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="52" t="n">
-        <v>46045.39704861111</v>
-      </c>
-      <c r="C7" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Schmidt</t>
-        </is>
-      </c>
-      <c r="D7" s="53" t="inlineStr">
-        <is>
-          <t>Reko Protokoll funktioniert, kein stabiler Prozess</t>
-        </is>
-      </c>
-      <c r="E7" s="52" t="n">
-        <v>46049.33333333334</v>
-      </c>
-      <c r="F7" s="51" t="inlineStr">
-        <is>
-          <t>Siebert</t>
-        </is>
-      </c>
-      <c r="G7" s="53" t="inlineStr">
-        <is>
-          <t>Speicher Geupdated, der Indexer muss noch ein Fehler behoben werden, in arbeit.</t>
-        </is>
-      </c>
+    <row r="5">
+      <c r="A5" s="51">
+        <f>IF(B5&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B5" s="52" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="52" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="53" t="n"/>
+      <c r="H5" s="52" t="n"/>
+      <c r="I5" s="51" t="n"/>
+      <c r="J5" s="51" t="n"/>
+      <c r="K5" s="53" t="n"/>
+      <c r="L5" s="53" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="51">
+        <f>IF(B6&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B6" s="52" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="53" t="n"/>
+      <c r="E6" s="52" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="53" t="n"/>
+      <c r="H6" s="52" t="n"/>
+      <c r="I6" s="51" t="n"/>
+      <c r="J6" s="51" t="n"/>
+      <c r="K6" s="53" t="n"/>
+      <c r="L6" s="53" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="51">
+        <f>IF(B7&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B7" s="52" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="53" t="n"/>
+      <c r="E7" s="52" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="53" t="n"/>
       <c r="H7" s="52" t="n"/>
-      <c r="I7" s="51" t="inlineStr"/>
-      <c r="J7" s="54" t="inlineStr"/>
-      <c r="K7" s="53" t="inlineStr"/>
-      <c r="L7" s="53" t="inlineStr"/>
+      <c r="I7" s="51" t="n"/>
+      <c r="J7" s="51" t="n"/>
+      <c r="K7" s="53" t="n"/>
+      <c r="L7" s="53" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="51">
@@ -8347,59 +7120,8 @@
       <c r="K54" s="53" t="n"/>
       <c r="L54" s="53" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="51">
-        <f>IF(B55&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="52" t="n"/>
-      <c r="C55" s="51" t="n"/>
-      <c r="D55" s="53" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="51" t="n"/>
-      <c r="J55" s="51" t="n"/>
-      <c r="K55" s="53" t="n"/>
-      <c r="L55" s="53" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="51">
-        <f>IF(B56&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B56" s="52" t="n"/>
-      <c r="C56" s="51" t="n"/>
-      <c r="D56" s="53" t="n"/>
-      <c r="E56" s="52" t="n"/>
-      <c r="F56" s="51" t="n"/>
-      <c r="G56" s="53" t="n"/>
-      <c r="H56" s="52" t="n"/>
-      <c r="I56" s="51" t="n"/>
-      <c r="J56" s="51" t="n"/>
-      <c r="K56" s="53" t="n"/>
-      <c r="L56" s="53" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="51">
-        <f>IF(B57&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B57" s="52" t="n"/>
-      <c r="C57" s="51" t="n"/>
-      <c r="D57" s="53" t="n"/>
-      <c r="E57" s="52" t="n"/>
-      <c r="F57" s="51" t="n"/>
-      <c r="G57" s="53" t="n"/>
-      <c r="H57" s="52" t="n"/>
-      <c r="I57" s="51" t="n"/>
-      <c r="J57" s="51" t="n"/>
-      <c r="K57" s="53" t="n"/>
-      <c r="L57" s="53" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L57"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
@@ -8470,7 +7192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L57"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -8605,105 +7327,56 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="52" t="n">
-        <v>45901.47143518519</v>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Schmidt</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>Antibiotika sind teilweise abgelaufen, nicht geordnet gelagert</t>
-        </is>
-      </c>
+    <row r="5">
+      <c r="A5" s="51">
+        <f>IF(B5&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B5" s="52" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="53" t="n"/>
       <c r="E5" s="52" t="n"/>
-      <c r="F5" s="51" t="inlineStr"/>
-      <c r="G5" s="53" t="inlineStr">
-        <is>
-          <t>Es wurde ein Verfalls Tabelle angelegt an der Innenseite des Schranks die Monatlich kontrolliert wird</t>
-        </is>
-      </c>
-      <c r="H5" s="52" t="n">
-        <v>45926.45503472222</v>
-      </c>
-      <c r="I5" s="51" t="inlineStr">
-        <is>
-          <t>Siebert</t>
-        </is>
-      </c>
-      <c r="J5" s="54" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="K5" s="53" t="inlineStr"/>
-      <c r="L5" s="53" t="inlineStr">
-        <is>
-          <t>Besprochen mit  Dr.Schmidt</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="52" t="n">
-        <v>46006.69575231482</v>
-      </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>Dr. Vitez</t>
-        </is>
-      </c>
-      <c r="D6" s="53" t="inlineStr">
-        <is>
-          <t>Hepatitis A-Impfstoff (Havrix) in November abgelaufen</t>
-        </is>
-      </c>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="53" t="n"/>
+      <c r="H5" s="52" t="n"/>
+      <c r="I5" s="51" t="n"/>
+      <c r="J5" s="51" t="n"/>
+      <c r="K5" s="53" t="n"/>
+      <c r="L5" s="53" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="51">
+        <f>IF(B6&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B6" s="52" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="53" t="n"/>
       <c r="E6" s="52" t="n"/>
-      <c r="F6" s="51" t="inlineStr"/>
-      <c r="G6" s="53" t="inlineStr"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="53" t="n"/>
       <c r="H6" s="52" t="n"/>
-      <c r="I6" s="51" t="inlineStr"/>
-      <c r="J6" s="54" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="K6" s="53" t="inlineStr"/>
-      <c r="L6" s="53" t="inlineStr"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="52" t="n">
-        <v>46045.39913194445</v>
-      </c>
-      <c r="C7" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Schmidt</t>
-        </is>
-      </c>
-      <c r="D7" s="53" t="inlineStr">
-        <is>
-          <t>Einträge (siehe 15.12.25) in diesem Bereich werden nicht rückgemeldet bzw. abgearbeitet</t>
-        </is>
-      </c>
+      <c r="I6" s="51" t="n"/>
+      <c r="J6" s="51" t="n"/>
+      <c r="K6" s="53" t="n"/>
+      <c r="L6" s="53" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="51">
+        <f>IF(B7&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B7" s="52" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="53" t="n"/>
       <c r="E7" s="52" t="n"/>
-      <c r="F7" s="51" t="inlineStr"/>
-      <c r="G7" s="53" t="inlineStr"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="53" t="n"/>
       <c r="H7" s="52" t="n"/>
-      <c r="I7" s="51" t="inlineStr"/>
-      <c r="J7" s="54" t="inlineStr"/>
-      <c r="K7" s="53" t="inlineStr"/>
-      <c r="L7" s="53" t="inlineStr"/>
+      <c r="I7" s="51" t="n"/>
+      <c r="J7" s="51" t="n"/>
+      <c r="K7" s="53" t="n"/>
+      <c r="L7" s="53" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="51">
@@ -9504,59 +8177,8 @@
       <c r="K54" s="53" t="n"/>
       <c r="L54" s="53" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="51">
-        <f>IF(B55&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="52" t="n"/>
-      <c r="C55" s="51" t="n"/>
-      <c r="D55" s="53" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="51" t="n"/>
-      <c r="J55" s="51" t="n"/>
-      <c r="K55" s="53" t="n"/>
-      <c r="L55" s="53" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="51">
-        <f>IF(B56&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B56" s="52" t="n"/>
-      <c r="C56" s="51" t="n"/>
-      <c r="D56" s="53" t="n"/>
-      <c r="E56" s="52" t="n"/>
-      <c r="F56" s="51" t="n"/>
-      <c r="G56" s="53" t="n"/>
-      <c r="H56" s="52" t="n"/>
-      <c r="I56" s="51" t="n"/>
-      <c r="J56" s="51" t="n"/>
-      <c r="K56" s="53" t="n"/>
-      <c r="L56" s="53" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="51">
-        <f>IF(B57&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B57" s="52" t="n"/>
-      <c r="C57" s="51" t="n"/>
-      <c r="D57" s="53" t="n"/>
-      <c r="E57" s="52" t="n"/>
-      <c r="F57" s="51" t="n"/>
-      <c r="G57" s="53" t="n"/>
-      <c r="H57" s="52" t="n"/>
-      <c r="I57" s="51" t="n"/>
-      <c r="J57" s="51" t="n"/>
-      <c r="K57" s="53" t="n"/>
-      <c r="L57" s="53" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L57"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
@@ -9627,7 +8249,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L56"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -9762,61 +8384,39 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="52" t="n">
-        <v>45974.37909722222</v>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
-        <is>
-          <t>Zuber</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>Barduschwäsche nur Herren raus gestellt, Damen volle Kiste stehen lassen</t>
-        </is>
-      </c>
+    <row r="5">
+      <c r="A5" s="51">
+        <f>IF(B5&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B5" s="52" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="53" t="n"/>
       <c r="E5" s="52" t="n"/>
-      <c r="F5" s="51" t="inlineStr"/>
-      <c r="G5" s="53" t="inlineStr"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="53" t="n"/>
       <c r="H5" s="52" t="n"/>
-      <c r="I5" s="51" t="inlineStr"/>
-      <c r="J5" s="54" t="inlineStr"/>
-      <c r="K5" s="53" t="inlineStr"/>
-      <c r="L5" s="53" t="inlineStr"/>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="52" t="n">
-        <v>46056.33333333334</v>
-      </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="D6" s="53" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
+      <c r="I5" s="51" t="n"/>
+      <c r="J5" s="51" t="n"/>
+      <c r="K5" s="53" t="n"/>
+      <c r="L5" s="53" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="51">
+        <f>IF(B6&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B6" s="52" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="53" t="n"/>
       <c r="E6" s="52" t="n"/>
-      <c r="F6" s="51" t="inlineStr"/>
-      <c r="G6" s="53" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="53" t="n"/>
       <c r="H6" s="52" t="n"/>
-      <c r="I6" s="51" t="inlineStr"/>
-      <c r="J6" s="54" t="inlineStr"/>
-      <c r="K6" s="53" t="inlineStr"/>
-      <c r="L6" s="53" t="inlineStr"/>
+      <c r="I6" s="51" t="n"/>
+      <c r="J6" s="51" t="n"/>
+      <c r="K6" s="53" t="n"/>
+      <c r="L6" s="53" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="51">
@@ -10634,42 +9234,8 @@
       <c r="K54" s="53" t="n"/>
       <c r="L54" s="53" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="51">
-        <f>IF(B55&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="52" t="n"/>
-      <c r="C55" s="51" t="n"/>
-      <c r="D55" s="53" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="51" t="n"/>
-      <c r="J55" s="51" t="n"/>
-      <c r="K55" s="53" t="n"/>
-      <c r="L55" s="53" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="51">
-        <f>IF(B56&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B56" s="52" t="n"/>
-      <c r="C56" s="51" t="n"/>
-      <c r="D56" s="53" t="n"/>
-      <c r="E56" s="52" t="n"/>
-      <c r="F56" s="51" t="n"/>
-      <c r="G56" s="53" t="n"/>
-      <c r="H56" s="52" t="n"/>
-      <c r="I56" s="51" t="n"/>
-      <c r="J56" s="51" t="n"/>
-      <c r="K56" s="53" t="n"/>
-      <c r="L56" s="53" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L56"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
@@ -10740,7 +9306,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -10804,7 +9370,7 @@
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="49" t="inlineStr">
         <is>
-          <t>✉ Mail an Bereichsleiter: Goepfrich (Markus.Goepfrich@mercedes-benz.com)</t>
+          <t>✉ Mail an Bereichsleiter: Göpfrich (Markus.Goepfrich@mercedes-benz.com)</t>
         </is>
       </c>
       <c r="H3" s="50" t="inlineStr">
@@ -10875,237 +9441,90 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="52" t="n">
-        <v>45841.20189814815</v>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
-        <is>
-          <t>Breig</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>OP-Leuchte in Ambulanz 1 defekt</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="n">
-        <v>45889.71761574074</v>
-      </c>
-      <c r="F5" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="G5" s="53" t="inlineStr">
-        <is>
-          <t>Reperatur durch Reposition der Halterung (Dr. Frei)</t>
-        </is>
-      </c>
-      <c r="H5" s="52" t="n">
-        <v>45889.71751157408</v>
-      </c>
-      <c r="I5" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="J5" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K5" s="53" t="inlineStr"/>
-      <c r="L5" s="53" t="inlineStr">
-        <is>
-          <t>Besprochen mit  Dr.Frei</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="52" t="n">
-        <v>45910.91456018519</v>
-      </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>Wunsch</t>
-        </is>
-      </c>
-      <c r="D6" s="53" t="inlineStr">
-        <is>
-          <t>RR Manschette C3 aus dem RTW defekt, Leitung abgelöst durch MA der WF</t>
-        </is>
-      </c>
-      <c r="E6" s="52" t="n">
-        <v>45913.26006944444</v>
-      </c>
-      <c r="F6" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="G6" s="53" t="inlineStr">
-        <is>
-          <t>Neuteil am 24.09. erhalten u. eingeräumt. Zwischenzeitlich Nutzung d. RR-Manschette C3 KU.</t>
-        </is>
-      </c>
-      <c r="H6" s="52" t="n">
-        <v>45924.47547453704</v>
-      </c>
-      <c r="I6" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="J6" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K6" s="53" t="inlineStr"/>
-      <c r="L6" s="53" t="inlineStr">
-        <is>
-          <t>Besprochen mit  Dr.Schmidt</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="52" t="n">
-        <v>45912.17185185185</v>
-      </c>
-      <c r="C7" s="51" t="inlineStr">
-        <is>
-          <t>Zuber</t>
-        </is>
-      </c>
-      <c r="D7" s="53" t="inlineStr">
-        <is>
-          <t>Fehlendes Sperrlager für defekte Medizinprodukte, Defekte RR Manschette vom 10.09. kann nicht entsprechend hinterlegt werden. Bitte Sperrlager definieren und kommunizieren.</t>
-        </is>
-      </c>
-      <c r="E7" s="52" t="n">
-        <v>45913.26009259259</v>
-      </c>
-      <c r="F7" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="G7" s="53" t="inlineStr">
-        <is>
-          <t>Einrichtung eines Sperrlagers für defekte Medizinprodukte u. -geräte in Physikalische Therapie im 029/10 Schrank 2.</t>
-        </is>
-      </c>
-      <c r="H7" s="52" t="n">
-        <v>45954.88721064815</v>
-      </c>
-      <c r="I7" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="J7" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K7" s="53" t="inlineStr"/>
-      <c r="L7" s="53" t="inlineStr">
-        <is>
-          <t>Besprochen mit  Zuber</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="51" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="52" t="n">
-        <v>45967</v>
-      </c>
-      <c r="C8" s="51" t="inlineStr">
-        <is>
-          <t>Krempl</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr">
-        <is>
-          <t>Cryo-Thermal Gerät im WD Kuppenheim lässt sich nicht hochfahren, Bildschirm bleibt schwarz</t>
-        </is>
-      </c>
-      <c r="E8" s="52" t="n">
-        <v>45995.64162037037</v>
-      </c>
-      <c r="F8" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="G8" s="53" t="inlineStr">
-        <is>
-          <t>Reparatur durch Hersteller</t>
-        </is>
-      </c>
-      <c r="H8" s="52" t="n">
-        <v>46050.17486111111</v>
-      </c>
-      <c r="I8" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="J8" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K8" s="53" t="inlineStr"/>
-      <c r="L8" s="53" t="inlineStr">
-        <is>
-          <t>Besprochen mit  Dr.Frei</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="52" t="n">
-        <v>45995.64193287037</v>
-      </c>
-      <c r="C9" s="51" t="inlineStr">
-        <is>
-          <t>Göpfrich</t>
-        </is>
-      </c>
-      <c r="D9" s="53" t="inlineStr">
-        <is>
-          <t>Untersuchungsleuchte Ambulanz 1 defekt, Befestigung Lampenkopf gebrochen</t>
-        </is>
-      </c>
-      <c r="E9" s="52" t="n">
-        <v>45995.64219907407</v>
-      </c>
-      <c r="F9" s="51" t="inlineStr">
-        <is>
-          <t>Goepfrich</t>
-        </is>
-      </c>
-      <c r="G9" s="53" t="inlineStr"/>
+    <row r="5">
+      <c r="A5" s="51">
+        <f>IF(B5&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B5" s="52" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="52" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="53" t="n"/>
+      <c r="H5" s="52" t="n"/>
+      <c r="I5" s="51" t="n"/>
+      <c r="J5" s="51" t="n"/>
+      <c r="K5" s="53" t="n"/>
+      <c r="L5" s="53" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="51">
+        <f>IF(B6&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B6" s="52" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="53" t="n"/>
+      <c r="E6" s="52" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="53" t="n"/>
+      <c r="H6" s="52" t="n"/>
+      <c r="I6" s="51" t="n"/>
+      <c r="J6" s="51" t="n"/>
+      <c r="K6" s="53" t="n"/>
+      <c r="L6" s="53" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="51">
+        <f>IF(B7&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B7" s="52" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="53" t="n"/>
+      <c r="E7" s="52" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="53" t="n"/>
+      <c r="H7" s="52" t="n"/>
+      <c r="I7" s="51" t="n"/>
+      <c r="J7" s="51" t="n"/>
+      <c r="K7" s="53" t="n"/>
+      <c r="L7" s="53" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="51">
+        <f>IF(B8&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B8" s="52" t="n"/>
+      <c r="C8" s="51" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="52" t="n"/>
+      <c r="F8" s="51" t="n"/>
+      <c r="G8" s="53" t="n"/>
+      <c r="H8" s="52" t="n"/>
+      <c r="I8" s="51" t="n"/>
+      <c r="J8" s="51" t="n"/>
+      <c r="K8" s="53" t="n"/>
+      <c r="L8" s="53" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="51">
+        <f>IF(B9&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B9" s="52" t="n"/>
+      <c r="C9" s="51" t="n"/>
+      <c r="D9" s="53" t="n"/>
+      <c r="E9" s="52" t="n"/>
+      <c r="F9" s="51" t="n"/>
+      <c r="G9" s="53" t="n"/>
       <c r="H9" s="52" t="n"/>
-      <c r="I9" s="51" t="inlineStr"/>
-      <c r="J9" s="54" t="inlineStr"/>
-      <c r="K9" s="53" t="inlineStr"/>
-      <c r="L9" s="53" t="inlineStr"/>
+      <c r="I9" s="51" t="n"/>
+      <c r="J9" s="51" t="n"/>
+      <c r="K9" s="53" t="n"/>
+      <c r="L9" s="53" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="51">
@@ -11872,93 +10291,8 @@
       <c r="K54" s="53" t="n"/>
       <c r="L54" s="53" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="51">
-        <f>IF(B55&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="52" t="n"/>
-      <c r="C55" s="51" t="n"/>
-      <c r="D55" s="53" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="51" t="n"/>
-      <c r="J55" s="51" t="n"/>
-      <c r="K55" s="53" t="n"/>
-      <c r="L55" s="53" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="51">
-        <f>IF(B56&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B56" s="52" t="n"/>
-      <c r="C56" s="51" t="n"/>
-      <c r="D56" s="53" t="n"/>
-      <c r="E56" s="52" t="n"/>
-      <c r="F56" s="51" t="n"/>
-      <c r="G56" s="53" t="n"/>
-      <c r="H56" s="52" t="n"/>
-      <c r="I56" s="51" t="n"/>
-      <c r="J56" s="51" t="n"/>
-      <c r="K56" s="53" t="n"/>
-      <c r="L56" s="53" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="51">
-        <f>IF(B57&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B57" s="52" t="n"/>
-      <c r="C57" s="51" t="n"/>
-      <c r="D57" s="53" t="n"/>
-      <c r="E57" s="52" t="n"/>
-      <c r="F57" s="51" t="n"/>
-      <c r="G57" s="53" t="n"/>
-      <c r="H57" s="52" t="n"/>
-      <c r="I57" s="51" t="n"/>
-      <c r="J57" s="51" t="n"/>
-      <c r="K57" s="53" t="n"/>
-      <c r="L57" s="53" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="51">
-        <f>IF(B58&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B58" s="52" t="n"/>
-      <c r="C58" s="51" t="n"/>
-      <c r="D58" s="53" t="n"/>
-      <c r="E58" s="52" t="n"/>
-      <c r="F58" s="51" t="n"/>
-      <c r="G58" s="53" t="n"/>
-      <c r="H58" s="52" t="n"/>
-      <c r="I58" s="51" t="n"/>
-      <c r="J58" s="51" t="n"/>
-      <c r="K58" s="53" t="n"/>
-      <c r="L58" s="53" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="51">
-        <f>IF(B59&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B59" s="52" t="n"/>
-      <c r="C59" s="51" t="n"/>
-      <c r="D59" s="53" t="n"/>
-      <c r="E59" s="52" t="n"/>
-      <c r="F59" s="51" t="n"/>
-      <c r="G59" s="53" t="n"/>
-      <c r="H59" s="52" t="n"/>
-      <c r="I59" s="51" t="n"/>
-      <c r="J59" s="51" t="n"/>
-      <c r="K59" s="53" t="n"/>
-      <c r="L59" s="53" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L59"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
@@ -12029,7 +10363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L55"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -12164,51 +10498,22 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="52" t="n">
-        <v>45888.45252314815</v>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>EDTA Röhrchen vom 18.8. (K'heim) wurden in Rastatt nach dem Zentrifugieren in den Kühlschrank gelegt</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="n">
-        <v>45888.45719907407</v>
-      </c>
-      <c r="F5" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="G5" s="53" t="inlineStr">
-        <is>
-          <t>Rücksprache mit Labor; neue Verfahrensanweisung verschickt und visualisiert</t>
-        </is>
-      </c>
-      <c r="H5" s="52" t="n">
-        <v>45888.46002314815</v>
-      </c>
-      <c r="I5" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="J5" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K5" s="53" t="inlineStr"/>
-      <c r="L5" s="53" t="inlineStr"/>
+    <row r="5">
+      <c r="A5" s="51">
+        <f>IF(B5&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B5" s="52" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="52" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="53" t="n"/>
+      <c r="H5" s="52" t="n"/>
+      <c r="I5" s="51" t="n"/>
+      <c r="J5" s="51" t="n"/>
+      <c r="K5" s="53" t="n"/>
+      <c r="L5" s="53" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="51">
@@ -13043,25 +11348,8 @@
       <c r="K54" s="53" t="n"/>
       <c r="L54" s="53" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="51">
-        <f>IF(B55&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="52" t="n"/>
-      <c r="C55" s="51" t="n"/>
-      <c r="D55" s="53" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="51" t="n"/>
-      <c r="J55" s="51" t="n"/>
-      <c r="K55" s="53" t="n"/>
-      <c r="L55" s="53" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L55"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>
@@ -13132,7 +11420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L60"/>
+  <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -13267,253 +11555,107 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="51" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="52" t="n">
-        <v>45901.46358796296</v>
-      </c>
-      <c r="C5" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Schmidt</t>
-        </is>
-      </c>
-      <c r="D5" s="53" t="inlineStr">
-        <is>
-          <t>Laris Eintrag für Bereich bei EDV nicht möglich, obwohl Einträge in Bereichen zB Sekretariat/Mail und an Bereichsleiter möglich sind</t>
-        </is>
-      </c>
-      <c r="E5" s="52" t="n">
-        <v>45922</v>
-      </c>
-      <c r="F5" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="G5" s="53" t="inlineStr">
-        <is>
-          <t>Info an Harry Zuber--&gt; Bitte Fehler prüfen und beheben</t>
-        </is>
-      </c>
+    <row r="5">
+      <c r="A5" s="51">
+        <f>IF(B5&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B5" s="52" t="n"/>
+      <c r="C5" s="51" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="52" t="n"/>
+      <c r="F5" s="51" t="n"/>
+      <c r="G5" s="53" t="n"/>
       <c r="H5" s="52" t="n"/>
-      <c r="I5" s="51" t="inlineStr"/>
-      <c r="J5" s="54" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="K5" s="53" t="inlineStr"/>
-      <c r="L5" s="53" t="inlineStr"/>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="51" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="52" t="n">
-        <v>45901.47094907407</v>
-      </c>
-      <c r="C6" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Schmidt</t>
-        </is>
-      </c>
-      <c r="D6" s="53" t="inlineStr">
-        <is>
-          <t>Bereich Med. &amp; Verbr.: Antibiotika sind teilweise abgelaufen, nicht geordnet gelagert; hier Laris Eintrag nicht möglich, obwohl Einträge in Bereichen zB Sekretariat/Mail und an Bereichsleiter möglich sind</t>
-        </is>
-      </c>
-      <c r="E6" s="52" t="n">
-        <v>45902</v>
-      </c>
-      <c r="F6" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="G6" s="53" t="inlineStr">
-        <is>
-          <t>Bereichverantwortlicher hat Fehler abgestellt</t>
-        </is>
-      </c>
-      <c r="H6" s="52" t="n">
-        <v>45904</v>
-      </c>
-      <c r="I6" s="51" t="inlineStr">
-        <is>
-          <t>Siebert</t>
-        </is>
-      </c>
-      <c r="J6" s="54" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="K6" s="53" t="inlineStr"/>
-      <c r="L6" s="53" t="inlineStr"/>
-    </row>
-    <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="51" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="52" t="n">
-        <v>45923.37097222222</v>
-      </c>
-      <c r="C7" s="51" t="inlineStr">
-        <is>
-          <t>Dr.Schmidt</t>
-        </is>
-      </c>
-      <c r="D7" s="53" t="inlineStr">
-        <is>
-          <t>Dokument für Einverständniserklärung Blutabnahme wurden in falsche Akte gescannt</t>
-        </is>
-      </c>
-      <c r="E7" s="52" t="n">
-        <v>45923</v>
-      </c>
-      <c r="F7" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="G7" s="53" t="inlineStr">
-        <is>
-          <t>Fehler durch Sekretariat erkannt und behoben</t>
-        </is>
-      </c>
-      <c r="H7" s="52" t="n">
-        <v>45923</v>
-      </c>
-      <c r="I7" s="51" t="inlineStr">
-        <is>
-          <t>Radimersky</t>
-        </is>
-      </c>
-      <c r="J7" s="54" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="K7" s="53" t="inlineStr"/>
-      <c r="L7" s="53" t="inlineStr"/>
-    </row>
-    <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="51" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="52" t="n">
-        <v>45923.66394675926</v>
-      </c>
-      <c r="C8" s="51" t="inlineStr">
-        <is>
-          <t>Krempl</t>
-        </is>
-      </c>
-      <c r="D8" s="53" t="inlineStr">
-        <is>
-          <t>Glucoseröhrchen wurden über Nacht nicht gekühlt, dafür aber nicht die EDTA-Röhrchen die am Vortag aus Kuppenheim gebracht wurden.</t>
-        </is>
-      </c>
-      <c r="E8" s="52" t="n">
-        <v>45924</v>
-      </c>
-      <c r="F8" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="G8" s="53" t="inlineStr">
-        <is>
-          <t>Laborergebnis wird abgewartet; bei Abweichung werden die betreffenden Patienten erneut einbestellt</t>
-        </is>
-      </c>
-      <c r="H8" s="52" t="n">
-        <v>45924</v>
-      </c>
-      <c r="I8" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="J8" s="54" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="K8" s="53" t="inlineStr">
-        <is>
-          <t>Mit Mitarbeiter persönlich besprochen</t>
-        </is>
-      </c>
-      <c r="L8" s="53" t="inlineStr"/>
-    </row>
-    <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="51" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="52" t="n">
-        <v>45926.34351851852</v>
-      </c>
-      <c r="C9" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="D9" s="53" t="inlineStr">
-        <is>
-          <t>Serumröhrchen von drei Patienten aus Kuppenheim wurden am Vortag nicht aus der Zentrifuge genommen und waren 16 Stunden ungekühlt</t>
-        </is>
-      </c>
-      <c r="E9" s="52" t="n">
-        <v>45926.34329861111</v>
-      </c>
-      <c r="F9" s="51" t="inlineStr">
-        <is>
-          <t>Putschler</t>
-        </is>
-      </c>
-      <c r="G9" s="53" t="inlineStr">
-        <is>
-          <t>Serumröhrchen in den Kühlschrank getan; Rücksprache mit Arzt ob noch zu verwenden</t>
-        </is>
-      </c>
+      <c r="I5" s="51" t="n"/>
+      <c r="J5" s="51" t="n"/>
+      <c r="K5" s="53" t="n"/>
+      <c r="L5" s="53" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="51">
+        <f>IF(B6&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B6" s="52" t="n"/>
+      <c r="C6" s="51" t="n"/>
+      <c r="D6" s="53" t="n"/>
+      <c r="E6" s="52" t="n"/>
+      <c r="F6" s="51" t="n"/>
+      <c r="G6" s="53" t="n"/>
+      <c r="H6" s="52" t="n"/>
+      <c r="I6" s="51" t="n"/>
+      <c r="J6" s="51" t="n"/>
+      <c r="K6" s="53" t="n"/>
+      <c r="L6" s="53" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="51">
+        <f>IF(B7&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B7" s="52" t="n"/>
+      <c r="C7" s="51" t="n"/>
+      <c r="D7" s="53" t="n"/>
+      <c r="E7" s="52" t="n"/>
+      <c r="F7" s="51" t="n"/>
+      <c r="G7" s="53" t="n"/>
+      <c r="H7" s="52" t="n"/>
+      <c r="I7" s="51" t="n"/>
+      <c r="J7" s="51" t="n"/>
+      <c r="K7" s="53" t="n"/>
+      <c r="L7" s="53" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="51">
+        <f>IF(B8&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B8" s="52" t="n"/>
+      <c r="C8" s="51" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="52" t="n"/>
+      <c r="F8" s="51" t="n"/>
+      <c r="G8" s="53" t="n"/>
+      <c r="H8" s="52" t="n"/>
+      <c r="I8" s="51" t="n"/>
+      <c r="J8" s="51" t="n"/>
+      <c r="K8" s="53" t="n"/>
+      <c r="L8" s="53" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="51">
+        <f>IF(B9&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B9" s="52" t="n"/>
+      <c r="C9" s="51" t="n"/>
+      <c r="D9" s="53" t="n"/>
+      <c r="E9" s="52" t="n"/>
+      <c r="F9" s="51" t="n"/>
+      <c r="G9" s="53" t="n"/>
       <c r="H9" s="52" t="n"/>
-      <c r="I9" s="51" t="inlineStr"/>
-      <c r="J9" s="54" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="K9" s="53" t="inlineStr"/>
-      <c r="L9" s="53" t="inlineStr"/>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="51" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="52" t="n">
-        <v>45950.29810185185</v>
-      </c>
-      <c r="C10" s="51" t="inlineStr">
-        <is>
-          <t>Zuber</t>
-        </is>
-      </c>
-      <c r="D10" s="53" t="inlineStr">
-        <is>
-          <t>Testmeldung aus Qualitätsgründen</t>
-        </is>
-      </c>
+      <c r="I9" s="51" t="n"/>
+      <c r="J9" s="51" t="n"/>
+      <c r="K9" s="53" t="n"/>
+      <c r="L9" s="53" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="51">
+        <f>IF(B10&lt;&gt;"",ROW()-4,"")</f>
+        <v/>
+      </c>
+      <c r="B10" s="52" t="n"/>
+      <c r="C10" s="51" t="n"/>
+      <c r="D10" s="53" t="n"/>
       <c r="E10" s="52" t="n"/>
-      <c r="F10" s="51" t="inlineStr"/>
-      <c r="G10" s="53" t="inlineStr"/>
+      <c r="F10" s="51" t="n"/>
+      <c r="G10" s="53" t="n"/>
       <c r="H10" s="52" t="n"/>
-      <c r="I10" s="51" t="inlineStr"/>
-      <c r="J10" s="54" t="inlineStr"/>
-      <c r="K10" s="53" t="inlineStr"/>
-      <c r="L10" s="53" t="inlineStr"/>
+      <c r="I10" s="51" t="n"/>
+      <c r="J10" s="51" t="n"/>
+      <c r="K10" s="53" t="n"/>
+      <c r="L10" s="53" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="51">
@@ -14263,110 +12405,8 @@
       <c r="K54" s="53" t="n"/>
       <c r="L54" s="53" t="n"/>
     </row>
-    <row r="55">
-      <c r="A55" s="51">
-        <f>IF(B55&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B55" s="52" t="n"/>
-      <c r="C55" s="51" t="n"/>
-      <c r="D55" s="53" t="n"/>
-      <c r="E55" s="52" t="n"/>
-      <c r="F55" s="51" t="n"/>
-      <c r="G55" s="53" t="n"/>
-      <c r="H55" s="52" t="n"/>
-      <c r="I55" s="51" t="n"/>
-      <c r="J55" s="51" t="n"/>
-      <c r="K55" s="53" t="n"/>
-      <c r="L55" s="53" t="n"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="51">
-        <f>IF(B56&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B56" s="52" t="n"/>
-      <c r="C56" s="51" t="n"/>
-      <c r="D56" s="53" t="n"/>
-      <c r="E56" s="52" t="n"/>
-      <c r="F56" s="51" t="n"/>
-      <c r="G56" s="53" t="n"/>
-      <c r="H56" s="52" t="n"/>
-      <c r="I56" s="51" t="n"/>
-      <c r="J56" s="51" t="n"/>
-      <c r="K56" s="53" t="n"/>
-      <c r="L56" s="53" t="n"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="51">
-        <f>IF(B57&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B57" s="52" t="n"/>
-      <c r="C57" s="51" t="n"/>
-      <c r="D57" s="53" t="n"/>
-      <c r="E57" s="52" t="n"/>
-      <c r="F57" s="51" t="n"/>
-      <c r="G57" s="53" t="n"/>
-      <c r="H57" s="52" t="n"/>
-      <c r="I57" s="51" t="n"/>
-      <c r="J57" s="51" t="n"/>
-      <c r="K57" s="53" t="n"/>
-      <c r="L57" s="53" t="n"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="51">
-        <f>IF(B58&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B58" s="52" t="n"/>
-      <c r="C58" s="51" t="n"/>
-      <c r="D58" s="53" t="n"/>
-      <c r="E58" s="52" t="n"/>
-      <c r="F58" s="51" t="n"/>
-      <c r="G58" s="53" t="n"/>
-      <c r="H58" s="52" t="n"/>
-      <c r="I58" s="51" t="n"/>
-      <c r="J58" s="51" t="n"/>
-      <c r="K58" s="53" t="n"/>
-      <c r="L58" s="53" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="51">
-        <f>IF(B59&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B59" s="52" t="n"/>
-      <c r="C59" s="51" t="n"/>
-      <c r="D59" s="53" t="n"/>
-      <c r="E59" s="52" t="n"/>
-      <c r="F59" s="51" t="n"/>
-      <c r="G59" s="53" t="n"/>
-      <c r="H59" s="52" t="n"/>
-      <c r="I59" s="51" t="n"/>
-      <c r="J59" s="51" t="n"/>
-      <c r="K59" s="53" t="n"/>
-      <c r="L59" s="53" t="n"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="51">
-        <f>IF(B60&lt;&gt;"",ROW()-4,"")</f>
-        <v/>
-      </c>
-      <c r="B60" s="52" t="n"/>
-      <c r="C60" s="51" t="n"/>
-      <c r="D60" s="53" t="n"/>
-      <c r="E60" s="52" t="n"/>
-      <c r="F60" s="51" t="n"/>
-      <c r="G60" s="53" t="n"/>
-      <c r="H60" s="52" t="n"/>
-      <c r="I60" s="51" t="n"/>
-      <c r="J60" s="51" t="n"/>
-      <c r="K60" s="53" t="n"/>
-      <c r="L60" s="53" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A4:L60"/>
+  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="H3:L3"/>

</xml_diff>

<commit_message>
Dynamische Mail-Erinnerung statt VBA-Popup
Ersetzt das alte VBA Worksheet_Deactivate-Popup durch eine
formelbasierte Erinnerung in Zelle H3 jedes Bereichs-Sheets:
- Orange + "⚠ X Meldung(en) ohne Kenntnisnahme - Mail senden!"
  wenn Eintraege ohne Kenntnisnahme existieren
- Gruen + "✓ Alles bearbeitet" wenn alles abgearbeitet ist
- Nutzt COUNTIFS auf Meldung-am vs Kenntnisnahme-am Spalten

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/LARIS_2026.xlsx
+++ b/LARIS_2026.xlsx
@@ -53,7 +53,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD.MM.YYYY HH:MM"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="24">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -199,12 +199,6 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
       <u val="single"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <color rgb="00666666"/>
-      <sz val="9"/>
     </font>
   </fonts>
   <fills count="15">
@@ -456,7 +450,7 @@
     <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -516,7 +510,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="11">
+  <dxfs count="13">
     <dxf>
       <font>
         <b val="1"/>
@@ -570,6 +564,34 @@
         <patternFill patternType="solid">
           <fgColor rgb="00FFE0B2"/>
           <bgColor rgb="00FFE0B2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00FF6F00"/>
+          <bgColor rgb="00FF6F00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Calibri"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+        <sz val="11"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="0028A745"/>
+          <bgColor rgb="0028A745"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1767,10 +1789,9 @@
           <t>✉ Mail an: Zieger-Buchta (CC: Müller-Horn)</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler | CC: Müller-Horn</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -2693,43 +2714,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2840,10 +2869,9 @@
           <t>✉ Mail an: Wunsch</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -3766,43 +3794,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -5270,10 +5306,9 @@
           <t>✉ Mail an: Emily Schmidt (CC: Larissa Radimersky)</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler | CC: Larissa Radimersky</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -6196,43 +6231,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6343,10 +6386,9 @@
           <t>✉ Mail an: Siebert</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -7269,43 +7311,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7416,10 +7466,9 @@
           <t>✉ Mail an: Zeller (CC: Breig)</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler | CC: Breig</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -8342,43 +8391,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -8489,10 +8546,9 @@
           <t>✉ Mail an: Wunsch</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -9415,43 +9471,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -9562,10 +9626,9 @@
           <t>✉ Mail an: Göpfrich</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -10488,43 +10551,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10635,10 +10706,9 @@
           <t>✉ Mail an: Wunsch</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -11561,43 +11631,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11708,10 +11786,9 @@
           <t>✉ Mail an: Putschler</t>
         </is>
       </c>
-      <c r="H3" s="51" t="inlineStr">
-        <is>
-          <t>BCC: Putschler</t>
-        </is>
+      <c r="H3" s="51">
+        <f>IF(COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0,"⚠ "&amp;COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&amp;" Meldung(en) ohne Kenntnisnahme - Mail senden!","✓ Alles bearbeitet | BCC: Putschler")</f>
+        <v/>
       </c>
     </row>
     <row r="4" ht="32" customHeight="1">
@@ -12634,43 +12711,51 @@
     <mergeCell ref="H3:L3"/>
     <mergeCell ref="A3:G3"/>
   </mergeCells>
+  <conditionalFormatting sqref="H3">
+    <cfRule type="expression" priority="1" dxfId="6" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")&gt;0</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="7" stopIfTrue="1">
+      <formula>COUNTIFS(B5:B504,"&lt;&gt;",E5:E504,"")=0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="J5:J504">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="3" stopIfTrue="1">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3" stopIfTrue="1">
       <formula>"A"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="4" stopIfTrue="1">
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="4" stopIfTrue="1">
       <formula>"B"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="5" stopIfTrue="1">
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="5" stopIfTrue="1">
       <formula>"C"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="4" operator="equal" dxfId="2" stopIfTrue="1">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="2" stopIfTrue="1">
       <formula>"D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:L504">
-    <cfRule type="expression" priority="5" dxfId="6" stopIfTrue="0">
+    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5&lt;&gt;"")</formula>
     </cfRule>
-    <cfRule type="expression" priority="6" dxfId="7" stopIfTrue="0">
+    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",$H5="")</formula>
     </cfRule>
-    <cfRule type="expression" priority="7" dxfId="8" stopIfTrue="1">
+    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$E5="",(TODAY()-$B5)&gt;14)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A5:A504">
-    <cfRule type="expression" priority="8" dxfId="9" stopIfTrue="0">
+    <cfRule type="expression" priority="10" dxfId="11" stopIfTrue="0">
       <formula>AND($B5&lt;&gt;"",(TODAY()-$B5)&lt;=7)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:C504">
-    <cfRule type="expression" priority="9" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="11" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$C5="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D5:D504">
-    <cfRule type="expression" priority="10" dxfId="10" stopIfTrue="1">
+    <cfRule type="expression" priority="12" dxfId="12" stopIfTrue="1">
       <formula>AND($B5&lt;&gt;"",$D5="")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Remove auto-filter buttons from LARIS department sheets
The dropdown filter arrows on header cells were unnecessary clutter.

https://claude.ai/code/session_0143BHkUCZBxvBT1DPHnv3wk
</commit_message>
<xml_diff>
--- a/LARIS_2026.xlsx
+++ b/LARIS_2026.xlsx
@@ -25,23 +25,14 @@
     <definedName name="NamenListe">Hilfslisten!$F$23:$F$38</definedName>
     <definedName name="REKOListe">Hilfslisten!$H$23:$H$40</definedName>
     <definedName name="KatListe">Hilfslisten!$J$23:$J$26</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sekretariat'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Sekretariat'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'EDV'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'EDV'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Med.&amp;Verbr.-stoff'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Med.&amp;Verbr.-stoff'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'WD-Fzg &amp; Schutzkleidg'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'WD-Fzg &amp; Schutzkleidg'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'RTW &amp; MPG'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="6">'RTW &amp; MPG'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Organisation Ambulanz'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'Organisation Ambulanz'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Ablauf&amp;Prozessprobleme'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'Ablauf&amp;Prozessprobleme'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'BGF'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'BGF'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Hygiene'!$A$4:$L$54</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'Hygiene'!$4:$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2707,7 +2698,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -3787,7 +3777,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -6224,7 +6213,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -7304,7 +7292,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -8384,7 +8371,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -9464,7 +9450,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -10544,7 +10529,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -11624,7 +11608,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>
@@ -12704,7 +12687,6 @@
       <c r="L54" s="54" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L54"/>
   <mergeCells count="4">
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="A1:K1"/>

</xml_diff>